<commit_message>
Update closing lines: Poll done: 25 snapshotted, 0 finalized with vig, 0 missed pre-match Wrote 91 matches to data/closing_lines/valorant_closing_lines.xlsx
</commit_message>
<xml_diff>
--- a/data/closing_lines/valorant_closing_lines.xlsx
+++ b/data/closing_lines/valorant_closing_lines.xlsx
@@ -756,7 +756,7 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
@@ -854,10 +854,10 @@
         <v>0.8</v>
       </c>
       <c r="V3" t="n">
-        <v>0.7428516333872839</v>
+        <v>0.7432573286166072</v>
       </c>
       <c r="W3" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X3" t="b">
         <v>1</v>
@@ -967,10 +967,10 @@
         <v>0.4901960784313725</v>
       </c>
       <c r="V4" t="n">
-        <v>0.4551786969284827</v>
+        <v>0.4554272846915485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X4" t="b">
         <v>1</v>
@@ -1077,7 +1077,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
@@ -1187,10 +1187,10 @@
         <v>0.4975124378109453</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4619724088229378</v>
+        <v>0.4622247068511239</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X6" t="b">
         <v>1</v>
@@ -1389,10 +1389,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="V8" t="n">
-        <v>0.5627663889297605</v>
+        <v>0.56307373380046</v>
       </c>
       <c r="W8" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X8" t="b">
         <v>1</v>
@@ -1502,10 +1502,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="V9" t="n">
-        <v>0.7738037847784207</v>
+        <v>0.7742263839756325</v>
       </c>
       <c r="W9" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X9" t="b">
         <v>1</v>
@@ -1603,10 +1603,10 @@
         <v>0.6451612903225806</v>
       </c>
       <c r="V10" t="n">
-        <v>0.5990738978929708</v>
+        <v>0.5994010714650058</v>
       </c>
       <c r="W10" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X10" t="b">
         <v>1</v>
@@ -1716,10 +1716,10 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="V11" t="n">
-        <v>0.4574209565192635</v>
+        <v>0.4576707688525907</v>
       </c>
       <c r="W11" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
@@ -1829,10 +1829,10 @@
         <v>0.3802281368821293</v>
       </c>
       <c r="V12" t="n">
-        <v>0.3530663656783669</v>
+        <v>0.3532591866048513</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
@@ -2132,10 +2132,10 @@
         <v>0.6289308176100629</v>
       </c>
       <c r="V15" t="n">
-        <v>0.5840028564365438</v>
+        <v>0.5843217992268924</v>
       </c>
       <c r="W15" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X15" t="b">
         <v>1</v>
@@ -2346,10 +2346,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="V17" t="n">
-        <v>0.6190430278227365</v>
+        <v>0.619381107180506</v>
       </c>
       <c r="W17" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X17" t="b">
         <v>1</v>
@@ -2456,7 +2456,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
@@ -2566,10 +2566,10 @@
         <v>0.8928571428571428</v>
       </c>
       <c r="V19" t="n">
-        <v>0.8290754836911649</v>
+        <v>0.8295282685453205</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X19" t="b">
         <v>1</v>
@@ -2679,10 +2679,10 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="V20" t="n">
-        <v>0.4318904845274906</v>
+        <v>0.4321263538468647</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
@@ -2792,10 +2792,10 @@
         <v>0.4566210045662101</v>
       </c>
       <c r="V21" t="n">
-        <v>0.4240020738511894</v>
+        <v>0.4242336350551411</v>
       </c>
       <c r="W21" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
@@ -2905,10 +2905,10 @@
         <v>0.4694835680751174</v>
       </c>
       <c r="V22" t="n">
-        <v>0.4359457942413638</v>
+        <v>0.436183878296131</v>
       </c>
       <c r="W22" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
@@ -3018,10 +3018,10 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="V23" t="n">
-        <v>0.5696714979963833</v>
+        <v>0.5699826139697908</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X23" t="b">
         <v>1</v>
@@ -3131,10 +3131,10 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="V24" t="n">
-        <v>0.5306083095623455</v>
+        <v>0.5308980918690051</v>
       </c>
       <c r="W24" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X24" t="b">
         <v>1</v>
@@ -3244,10 +3244,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="V25" t="n">
-        <v>0.7738037847784207</v>
+        <v>0.7742263839756325</v>
       </c>
       <c r="W25" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X25" t="b">
         <v>1</v>
@@ -3357,10 +3357,10 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="V26" t="n">
-        <v>0.4380021423274079</v>
+        <v>0.4382413494201693</v>
       </c>
       <c r="W26" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
@@ -3470,10 +3470,10 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="V27" t="n">
-        <v>0.6448364873153505</v>
+        <v>0.645188653313027</v>
       </c>
       <c r="W27" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X27" t="b">
         <v>1</v>
@@ -3583,10 +3583,10 @@
         <v>0.3759398496240601</v>
       </c>
       <c r="V28" t="n">
-        <v>0.3490844141857536</v>
+        <v>0.3492750604401349</v>
       </c>
       <c r="W28" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X28" t="b">
         <v>1</v>
@@ -3696,10 +3696,10 @@
         <v>0.4629629629629629</v>
       </c>
       <c r="V29" t="n">
-        <v>0.429890991543567</v>
+        <v>0.4301257688753513</v>
       </c>
       <c r="W29" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X29" t="b">
         <v>1</v>
@@ -3809,10 +3809,10 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="V30" t="n">
-        <v>0.6274084741446654</v>
+        <v>0.6277511221424047</v>
       </c>
       <c r="W30" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X30" t="b">
         <v>1</v>
@@ -3922,10 +3922,10 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="V31" t="n">
-        <v>0.4913039903355053</v>
+        <v>0.491572307286116</v>
       </c>
       <c r="W31" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X31" t="b">
         <v>1</v>
@@ -4032,7 +4032,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X32" t="b">
         <v>1</v>
@@ -4142,10 +4142,10 @@
         <v>0.8</v>
       </c>
       <c r="V33" t="n">
-        <v>0.7428516333872839</v>
+        <v>0.7432573286166072</v>
       </c>
       <c r="W33" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X33" t="b">
         <v>1</v>
@@ -4356,10 +4356,10 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="V35" t="n">
-        <v>0.3934595515822478</v>
+        <v>0.3936744325299826</v>
       </c>
       <c r="W35" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X35" t="b">
         <v>1</v>
@@ -4469,10 +4469,10 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="V36" t="n">
-        <v>0.5876990770469017</v>
+        <v>0.5880200384625056</v>
       </c>
       <c r="W36" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X36" t="b">
         <v>1</v>
@@ -4772,10 +4772,10 @@
         <v>0.591715976331361</v>
       </c>
       <c r="V39" t="n">
-        <v>0.5494464743988786</v>
+        <v>0.5497465448347686</v>
       </c>
       <c r="W39" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X39" t="b">
         <v>1</v>
@@ -4986,10 +4986,10 @@
         <v>0.8064516129032259</v>
       </c>
       <c r="V41" t="n">
-        <v>0.7488423723662135</v>
+        <v>0.7492513393312573</v>
       </c>
       <c r="W41" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X41" t="b">
         <v>1</v>
@@ -5096,7 +5096,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X42" t="b">
         <v>1</v>
@@ -5203,7 +5203,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X43" t="b">
         <v>1</v>
@@ -5310,7 +5310,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X44" t="b">
         <v>1</v>
@@ -5420,10 +5420,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="V45" t="n">
-        <v>0.6190430278227365</v>
+        <v>0.619381107180506</v>
       </c>
       <c r="W45" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X45" t="b">
         <v>1</v>
@@ -5533,10 +5533,10 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="V46" t="n">
-        <v>0.4421735913019546</v>
+        <v>0.4424150765575042</v>
       </c>
       <c r="W46" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X46" t="b">
         <v>1</v>
@@ -5646,10 +5646,10 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="V47" t="n">
-        <v>0.3934595515822478</v>
+        <v>0.3936744325299826</v>
       </c>
       <c r="W47" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X47" t="b">
         <v>1</v>
@@ -5759,10 +5759,10 @@
         <v>0.5</v>
       </c>
       <c r="V48" t="n">
-        <v>0.4642822708670524</v>
+        <v>0.4645358303853795</v>
       </c>
       <c r="W48" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X48" t="b">
         <v>1</v>
@@ -5869,7 +5869,7 @@
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X49" t="b">
         <v>1</v>
@@ -6080,10 +6080,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="V51" t="n">
-        <v>0.5216654728843285</v>
+        <v>0.5219503712195276</v>
       </c>
       <c r="W51" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X51" t="b">
         <v>1</v>
@@ -6193,10 +6193,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="V52" t="n">
-        <v>0.5627663889297605</v>
+        <v>0.56307373380046</v>
       </c>
       <c r="W52" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X52" t="b">
         <v>1</v>
@@ -6306,10 +6306,10 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="V53" t="n">
-        <v>0.5462144363141793</v>
+        <v>0.5465127416298582</v>
       </c>
       <c r="W53" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X53" t="b">
         <v>1</v>
@@ -6419,10 +6419,10 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="V54" t="n">
-        <v>0.6149434051219237</v>
+        <v>0.6152792455435491</v>
       </c>
       <c r="W54" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X54" t="b">
         <v>1</v>
@@ -6532,10 +6532,10 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="V55" t="n">
-        <v>0.5914423832701304</v>
+        <v>0.5917653890259611</v>
       </c>
       <c r="W55" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X55" t="b">
         <v>1</v>
@@ -6645,10 +6645,10 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="V56" t="n">
-        <v>0.4318904845274906</v>
+        <v>0.4321263538468647</v>
       </c>
       <c r="W56" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X56" t="b">
         <v>1</v>
@@ -6758,10 +6758,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="V57" t="n">
-        <v>0.6981688283715073</v>
+        <v>0.6985501208802698</v>
       </c>
       <c r="W57" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X57" t="b">
         <v>1</v>
@@ -6871,10 +6871,10 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="V58" t="n">
-        <v>0.4574209565192635</v>
+        <v>0.4576707688525907</v>
       </c>
       <c r="W58" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X58" t="b">
         <v>1</v>
@@ -6984,10 +6984,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="V59" t="n">
-        <v>0.5767481625677668</v>
+        <v>0.5770631433358751</v>
       </c>
       <c r="W59" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X59" t="b">
         <v>1</v>
@@ -7097,10 +7097,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="V60" t="n">
-        <v>0.6981688283715073</v>
+        <v>0.6985501208802698</v>
       </c>
       <c r="W60" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X60" t="b">
         <v>1</v>
@@ -7207,7 +7207,7 @@
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X61" t="b">
         <v>1</v>
@@ -7418,10 +7418,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="V63" t="n">
-        <v>0.3869018923892104</v>
+        <v>0.3871131919878162</v>
       </c>
       <c r="W63" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X63" t="b">
         <v>1</v>
@@ -7531,10 +7531,10 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="V64" t="n">
-        <v>0.6777843370321932</v>
+        <v>0.6781544969129627</v>
       </c>
       <c r="W64" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X64" t="b">
         <v>1</v>
@@ -7641,7 +7641,7 @@
       <c r="U65" t="inlineStr"/>
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X65" t="b">
         <v>1</v>
@@ -7751,10 +7751,10 @@
         <v>0.3521126760563381</v>
       </c>
       <c r="V66" t="n">
-        <v>0.3269593456810228</v>
+        <v>0.3271379087220982</v>
       </c>
       <c r="W66" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X66" t="b">
         <v>1</v>
@@ -7864,10 +7864,10 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="V67" t="n">
-        <v>0.6493458333804929</v>
+        <v>0.6497004620774539</v>
       </c>
       <c r="W67" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X67" t="b">
         <v>1</v>
@@ -7977,10 +7977,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="V68" t="n">
-        <v>0.5767481625677668</v>
+        <v>0.5770631433358751</v>
       </c>
       <c r="W68" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X68" t="b">
         <v>1</v>
@@ -8087,7 +8087,7 @@
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
       <c r="W69" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X69" t="b">
         <v>1</v>
@@ -8197,10 +8197,10 @@
         <v>0.8547008547008548</v>
       </c>
       <c r="V70" t="n">
-        <v>0.7936449074650469</v>
+        <v>0.7940783425391102</v>
       </c>
       <c r="W70" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X70" t="b">
         <v>1</v>
@@ -8310,10 +8310,10 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="V71" t="n">
-        <v>0.6585564125773793</v>
+        <v>0.6589160714686234</v>
       </c>
       <c r="W71" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X71" t="b">
         <v>1</v>
@@ -8423,10 +8423,10 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="V72" t="n">
-        <v>0.708827894453515</v>
+        <v>0.7092150082219534</v>
       </c>
       <c r="W72" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X72" t="b">
         <v>1</v>
@@ -8536,10 +8536,10 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="V73" t="n">
-        <v>0.5593762299603041</v>
+        <v>0.559681723355879</v>
       </c>
       <c r="W73" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X73" t="b">
         <v>1</v>
@@ -8649,10 +8649,10 @@
         <v>0.3731343283582089</v>
       </c>
       <c r="V74" t="n">
-        <v>0.3464793066172032</v>
+        <v>0.3466685301383429</v>
       </c>
       <c r="W74" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X74" t="b">
         <v>1</v>
@@ -8762,10 +8762,10 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="V75" t="n">
-        <v>0.6493458333804929</v>
+        <v>0.6497004620774539</v>
       </c>
       <c r="W75" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X75" t="b">
         <v>1</v>
@@ -8875,10 +8875,10 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="V76" t="n">
-        <v>0.7198174742124842</v>
+        <v>0.7202105897447744</v>
       </c>
       <c r="W76" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X76" t="b">
         <v>1</v>
@@ -8988,10 +8988,10 @@
         <v>0.8</v>
       </c>
       <c r="V77" t="n">
-        <v>0.7428516333872839</v>
+        <v>0.7432573286166072</v>
       </c>
       <c r="W77" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X77" t="b">
         <v>1</v>
@@ -9101,10 +9101,10 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="V78" t="n">
-        <v>0.5696714979963833</v>
+        <v>0.5699826139697908</v>
       </c>
       <c r="W78" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X78" t="b">
         <v>1</v>
@@ -9214,10 +9214,10 @@
         <v>0.8620689655172414</v>
       </c>
       <c r="V79" t="n">
-        <v>0.8004866739087111</v>
+        <v>0.8009238454920337</v>
       </c>
       <c r="W79" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X79" t="b">
         <v>1</v>
@@ -9327,10 +9327,10 @@
         <v>0.28328611898017</v>
       </c>
       <c r="V80" t="n">
-        <v>0.2630494452504546</v>
+        <v>0.2631931050342093</v>
       </c>
       <c r="W80" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X80" t="b">
         <v>1</v>
@@ -9437,7 +9437,7 @@
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr"/>
       <c r="W81" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X81" t="b">
         <v>1</v>
@@ -9547,10 +9547,10 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="V82" t="n">
-        <v>0.4380021423274079</v>
+        <v>0.4382413494201693</v>
       </c>
       <c r="W82" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X82" t="b">
         <v>1</v>
@@ -9660,10 +9660,10 @@
         <v>0.2702702702702702</v>
       </c>
       <c r="V83" t="n">
-        <v>0.2509633896578661</v>
+        <v>0.2511004488569619</v>
       </c>
       <c r="W83" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X83" t="b">
         <v>1</v>
@@ -9773,10 +9773,10 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="V84" t="n">
-        <v>0.383704356088473</v>
+        <v>0.3839139094094046</v>
       </c>
       <c r="W84" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X84" t="b">
         <v>1</v>
@@ -9883,7 +9883,7 @@
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="inlineStr"/>
       <c r="W85" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X85" t="b">
         <v>1</v>
@@ -9993,10 +9993,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="V86" t="n">
-        <v>0.5216654728843285</v>
+        <v>0.5219503712195276</v>
       </c>
       <c r="W86" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X86" t="b">
         <v>1</v>
@@ -10305,7 +10305,7 @@
       <c r="U89" t="inlineStr"/>
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X89" t="b">
         <v>1</v>
@@ -10415,10 +10415,10 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="V90" t="n">
-        <v>0.7549305217350445</v>
+        <v>0.7553428136347634</v>
       </c>
       <c r="W90" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X90" t="b">
         <v>1</v>
@@ -10528,10 +10528,10 @@
         <v>0.2932551319648093</v>
       </c>
       <c r="V91" t="n">
-        <v>0.2723063172240776</v>
+        <v>0.2724550324840935</v>
       </c>
       <c r="W91" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X91" t="b">
         <v>1</v>
@@ -10629,10 +10629,10 @@
         <v>0.53475935828877</v>
       </c>
       <c r="V92" t="n">
-        <v>0.4965585784674356</v>
+        <v>0.4968297651180528</v>
       </c>
       <c r="W92" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="X92" t="b">
         <v>1</v>
@@ -10888,7 +10888,7 @@
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z2" t="b">
         <v>1</v>
@@ -11060,13 +11060,13 @@
         <v>0.8</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z4" t="b">
         <v>1</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.7428516333872839</v>
+        <v>0.7432573286166072</v>
       </c>
     </row>
     <row r="5">
@@ -11234,13 +11234,13 @@
         <v>0.4901960784313725</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z6" t="b">
         <v>1</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.4551786969284827</v>
+        <v>0.4554272846915485</v>
       </c>
     </row>
     <row r="7">
@@ -11400,7 +11400,7 @@
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z8" t="b">
         <v>1</v>
@@ -11485,13 +11485,13 @@
         <v>0.4975124378109453</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z9" t="b">
         <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.4619724088229378</v>
+        <v>0.4622247068511239</v>
       </c>
     </row>
     <row r="10">
@@ -11746,13 +11746,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z12" t="b">
         <v>1</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.5627663889297605</v>
+        <v>0.56307373380046</v>
       </c>
     </row>
     <row r="13">
@@ -11833,13 +11833,13 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z13" t="b">
         <v>1</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.7738037847784207</v>
+        <v>0.7742263839756325</v>
       </c>
     </row>
     <row r="14">
@@ -12007,13 +12007,13 @@
         <v>0.6451612903225806</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z15" t="b">
         <v>1</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.5990738978929708</v>
+        <v>0.5994010714650058</v>
       </c>
     </row>
     <row r="16">
@@ -12181,13 +12181,13 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z17" t="b">
         <v>1</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.4574209565192635</v>
+        <v>0.4576707688525907</v>
       </c>
     </row>
     <row r="18">
@@ -12268,13 +12268,13 @@
         <v>0.3802281368821293</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z18" t="b">
         <v>1</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.3530663656783669</v>
+        <v>0.3532591866048513</v>
       </c>
     </row>
     <row r="19">
@@ -12616,13 +12616,13 @@
         <v>0.6289308176100629</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z22" t="b">
         <v>1</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.5840028564365438</v>
+        <v>0.5843217992268924</v>
       </c>
     </row>
     <row r="23">
@@ -12877,13 +12877,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z25" t="b">
         <v>1</v>
       </c>
       <c r="AA25" t="n">
-        <v>0.6190430278227365</v>
+        <v>0.619381107180506</v>
       </c>
     </row>
     <row r="26">
@@ -13043,7 +13043,7 @@
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z27" t="b">
         <v>1</v>
@@ -13215,13 +13215,13 @@
         <v>0.8928571428571428</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z29" t="b">
         <v>1</v>
       </c>
       <c r="AA29" t="n">
-        <v>0.8290754836911649</v>
+        <v>0.8295282685453205</v>
       </c>
     </row>
     <row r="30">
@@ -13389,13 +13389,13 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z31" t="b">
         <v>1</v>
       </c>
       <c r="AA31" t="n">
-        <v>0.4318904845274906</v>
+        <v>0.4321263538468647</v>
       </c>
     </row>
     <row r="32">
@@ -13563,13 +13563,13 @@
         <v>0.4566210045662101</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z33" t="b">
         <v>1</v>
       </c>
       <c r="AA33" t="n">
-        <v>0.4240020738511894</v>
+        <v>0.4242336350551411</v>
       </c>
     </row>
     <row r="34">
@@ -13737,13 +13737,13 @@
         <v>0.4694835680751174</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z35" t="b">
         <v>1</v>
       </c>
       <c r="AA35" t="n">
-        <v>0.4359457942413638</v>
+        <v>0.436183878296131</v>
       </c>
     </row>
     <row r="36">
@@ -13911,13 +13911,13 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z37" t="b">
         <v>1</v>
       </c>
       <c r="AA37" t="n">
-        <v>0.5696714979963833</v>
+        <v>0.5699826139697908</v>
       </c>
     </row>
     <row r="38">
@@ -14085,13 +14085,13 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z39" t="b">
         <v>1</v>
       </c>
       <c r="AA39" t="n">
-        <v>0.5306083095623455</v>
+        <v>0.5308980918690051</v>
       </c>
     </row>
     <row r="40">
@@ -14259,13 +14259,13 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z41" t="b">
         <v>1</v>
       </c>
       <c r="AA41" t="n">
-        <v>0.7738037847784207</v>
+        <v>0.7742263839756325</v>
       </c>
     </row>
     <row r="42">
@@ -14433,13 +14433,13 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z43" t="b">
         <v>1</v>
       </c>
       <c r="AA43" t="n">
-        <v>0.4380021423274079</v>
+        <v>0.4382413494201693</v>
       </c>
     </row>
     <row r="44">
@@ -14607,13 +14607,13 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z45" t="b">
         <v>1</v>
       </c>
       <c r="AA45" t="n">
-        <v>0.6448364873153505</v>
+        <v>0.645188653313027</v>
       </c>
     </row>
     <row r="46">
@@ -14781,13 +14781,13 @@
         <v>0.3759398496240601</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z47" t="b">
         <v>1</v>
       </c>
       <c r="AA47" t="n">
-        <v>0.3490844141857536</v>
+        <v>0.3492750604401349</v>
       </c>
     </row>
     <row r="48">
@@ -14955,13 +14955,13 @@
         <v>0.4629629629629629</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z49" t="b">
         <v>1</v>
       </c>
       <c r="AA49" t="n">
-        <v>0.429890991543567</v>
+        <v>0.4301257688753513</v>
       </c>
     </row>
     <row r="50">
@@ -15129,13 +15129,13 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z51" t="b">
         <v>1</v>
       </c>
       <c r="AA51" t="n">
-        <v>0.6274084741446654</v>
+        <v>0.6277511221424047</v>
       </c>
     </row>
     <row r="52">
@@ -15303,13 +15303,13 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z53" t="b">
         <v>1</v>
       </c>
       <c r="AA53" t="n">
-        <v>0.4913039903355053</v>
+        <v>0.491572307286116</v>
       </c>
     </row>
     <row r="54">
@@ -15469,7 +15469,7 @@
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr"/>
       <c r="Y55" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z55" t="b">
         <v>1</v>
@@ -15641,13 +15641,13 @@
         <v>0.8</v>
       </c>
       <c r="Y57" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z57" t="b">
         <v>1</v>
       </c>
       <c r="AA57" t="n">
-        <v>0.7428516333872839</v>
+        <v>0.7432573286166072</v>
       </c>
     </row>
     <row r="58">
@@ -15902,13 +15902,13 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="Y60" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z60" t="b">
         <v>1</v>
       </c>
       <c r="AA60" t="n">
-        <v>0.3934595515822478</v>
+        <v>0.3936744325299826</v>
       </c>
     </row>
     <row r="61">
@@ -15989,13 +15989,13 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z61" t="b">
         <v>1</v>
       </c>
       <c r="AA61" t="n">
-        <v>0.5876990770469017</v>
+        <v>0.5880200384625056</v>
       </c>
     </row>
     <row r="62">
@@ -16337,13 +16337,13 @@
         <v>0.591715976331361</v>
       </c>
       <c r="Y65" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z65" t="b">
         <v>1</v>
       </c>
       <c r="AA65" t="n">
-        <v>0.5494464743988786</v>
+        <v>0.5497465448347686</v>
       </c>
     </row>
     <row r="66">
@@ -16598,13 +16598,13 @@
         <v>0.8064516129032259</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z68" t="b">
         <v>1</v>
       </c>
       <c r="AA68" t="n">
-        <v>0.7488423723662135</v>
+        <v>0.7492513393312573</v>
       </c>
     </row>
     <row r="69">
@@ -16764,7 +16764,7 @@
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
       <c r="Y70" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z70" t="b">
         <v>1</v>
@@ -16928,7 +16928,7 @@
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr"/>
       <c r="Y72" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z72" t="b">
         <v>1</v>
@@ -17092,7 +17092,7 @@
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr"/>
       <c r="Y74" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z74" t="b">
         <v>1</v>
@@ -17264,13 +17264,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="Y76" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z76" t="b">
         <v>1</v>
       </c>
       <c r="AA76" t="n">
-        <v>0.6190430278227365</v>
+        <v>0.619381107180506</v>
       </c>
     </row>
     <row r="77">
@@ -17438,13 +17438,13 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="Y78" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z78" t="b">
         <v>1</v>
       </c>
       <c r="AA78" t="n">
-        <v>0.4421735913019546</v>
+        <v>0.4424150765575042</v>
       </c>
     </row>
     <row r="79">
@@ -17612,13 +17612,13 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z80" t="b">
         <v>1</v>
       </c>
       <c r="AA80" t="n">
-        <v>0.3934595515822478</v>
+        <v>0.3936744325299826</v>
       </c>
     </row>
     <row r="81">
@@ -17786,13 +17786,13 @@
         <v>0.5</v>
       </c>
       <c r="Y82" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z82" t="b">
         <v>1</v>
       </c>
       <c r="AA82" t="n">
-        <v>0.4642822708670524</v>
+        <v>0.4645358303853795</v>
       </c>
     </row>
     <row r="83">
@@ -17952,7 +17952,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr"/>
       <c r="Y84" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z84" t="b">
         <v>1</v>
@@ -18211,13 +18211,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y87" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z87" t="b">
         <v>1</v>
       </c>
       <c r="AA87" t="n">
-        <v>0.5216654728843285</v>
+        <v>0.5219503712195276</v>
       </c>
     </row>
     <row r="88">
@@ -18385,13 +18385,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z89" t="b">
         <v>1</v>
       </c>
       <c r="AA89" t="n">
-        <v>0.5627663889297605</v>
+        <v>0.56307373380046</v>
       </c>
     </row>
     <row r="90">
@@ -18559,13 +18559,13 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z91" t="b">
         <v>1</v>
       </c>
       <c r="AA91" t="n">
-        <v>0.5462144363141793</v>
+        <v>0.5465127416298582</v>
       </c>
     </row>
     <row r="92">
@@ -18733,13 +18733,13 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="Y93" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z93" t="b">
         <v>1</v>
       </c>
       <c r="AA93" t="n">
-        <v>0.6149434051219237</v>
+        <v>0.6152792455435491</v>
       </c>
     </row>
     <row r="94">
@@ -18907,13 +18907,13 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="Y95" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z95" t="b">
         <v>1</v>
       </c>
       <c r="AA95" t="n">
-        <v>0.5914423832701304</v>
+        <v>0.5917653890259611</v>
       </c>
     </row>
     <row r="96">
@@ -19081,13 +19081,13 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="Y97" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z97" t="b">
         <v>1</v>
       </c>
       <c r="AA97" t="n">
-        <v>0.4318904845274906</v>
+        <v>0.4321263538468647</v>
       </c>
     </row>
     <row r="98">
@@ -19255,13 +19255,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y99" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z99" t="b">
         <v>1</v>
       </c>
       <c r="AA99" t="n">
-        <v>0.6981688283715073</v>
+        <v>0.6985501208802698</v>
       </c>
     </row>
     <row r="100">
@@ -19429,13 +19429,13 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="Y101" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z101" t="b">
         <v>1</v>
       </c>
       <c r="AA101" t="n">
-        <v>0.4574209565192635</v>
+        <v>0.4576707688525907</v>
       </c>
     </row>
     <row r="102">
@@ -19603,13 +19603,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y103" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z103" t="b">
         <v>1</v>
       </c>
       <c r="AA103" t="n">
-        <v>0.5767481625677668</v>
+        <v>0.5770631433358751</v>
       </c>
     </row>
     <row r="104">
@@ -19777,13 +19777,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y105" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z105" t="b">
         <v>1</v>
       </c>
       <c r="AA105" t="n">
-        <v>0.6981688283715073</v>
+        <v>0.6985501208802698</v>
       </c>
     </row>
     <row r="106">
@@ -19943,7 +19943,7 @@
       <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr"/>
       <c r="Y107" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z107" t="b">
         <v>1</v>
@@ -20202,13 +20202,13 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="Y110" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z110" t="b">
         <v>1</v>
       </c>
       <c r="AA110" t="n">
-        <v>0.3869018923892104</v>
+        <v>0.3871131919878162</v>
       </c>
     </row>
     <row r="111">
@@ -20376,13 +20376,13 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="Y112" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z112" t="b">
         <v>1</v>
       </c>
       <c r="AA112" t="n">
-        <v>0.6777843370321932</v>
+        <v>0.6781544969129627</v>
       </c>
     </row>
     <row r="113">
@@ -20542,7 +20542,7 @@
       <c r="W114" t="inlineStr"/>
       <c r="X114" t="inlineStr"/>
       <c r="Y114" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z114" t="b">
         <v>1</v>
@@ -20714,13 +20714,13 @@
         <v>0.3521126760563381</v>
       </c>
       <c r="Y116" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z116" t="b">
         <v>1</v>
       </c>
       <c r="AA116" t="n">
-        <v>0.3269593456810228</v>
+        <v>0.3271379087220982</v>
       </c>
     </row>
     <row r="117">
@@ -20888,13 +20888,13 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="Y118" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z118" t="b">
         <v>1</v>
       </c>
       <c r="AA118" t="n">
-        <v>0.6493458333804929</v>
+        <v>0.6497004620774539</v>
       </c>
     </row>
     <row r="119">
@@ -21062,13 +21062,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y120" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z120" t="b">
         <v>1</v>
       </c>
       <c r="AA120" t="n">
-        <v>0.5767481625677668</v>
+        <v>0.5770631433358751</v>
       </c>
     </row>
     <row r="121">
@@ -21228,7 +21228,7 @@
       <c r="W122" t="inlineStr"/>
       <c r="X122" t="inlineStr"/>
       <c r="Y122" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z122" t="b">
         <v>1</v>
@@ -21400,13 +21400,13 @@
         <v>0.8547008547008548</v>
       </c>
       <c r="Y124" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z124" t="b">
         <v>1</v>
       </c>
       <c r="AA124" t="n">
-        <v>0.7936449074650469</v>
+        <v>0.7940783425391102</v>
       </c>
     </row>
     <row r="125">
@@ -21574,13 +21574,13 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="Y126" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z126" t="b">
         <v>1</v>
       </c>
       <c r="AA126" t="n">
-        <v>0.6585564125773793</v>
+        <v>0.6589160714686234</v>
       </c>
     </row>
     <row r="127">
@@ -21748,13 +21748,13 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="Y128" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z128" t="b">
         <v>1</v>
       </c>
       <c r="AA128" t="n">
-        <v>0.708827894453515</v>
+        <v>0.7092150082219534</v>
       </c>
     </row>
     <row r="129">
@@ -21922,13 +21922,13 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="Y130" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z130" t="b">
         <v>1</v>
       </c>
       <c r="AA130" t="n">
-        <v>0.5593762299603041</v>
+        <v>0.559681723355879</v>
       </c>
     </row>
     <row r="131">
@@ -22096,13 +22096,13 @@
         <v>0.3731343283582089</v>
       </c>
       <c r="Y132" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z132" t="b">
         <v>1</v>
       </c>
       <c r="AA132" t="n">
-        <v>0.3464793066172032</v>
+        <v>0.3466685301383429</v>
       </c>
     </row>
     <row r="133">
@@ -22270,13 +22270,13 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="Y134" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z134" t="b">
         <v>1</v>
       </c>
       <c r="AA134" t="n">
-        <v>0.6493458333804929</v>
+        <v>0.6497004620774539</v>
       </c>
     </row>
     <row r="135">
@@ -22444,13 +22444,13 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="Y136" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z136" t="b">
         <v>1</v>
       </c>
       <c r="AA136" t="n">
-        <v>0.7198174742124842</v>
+        <v>0.7202105897447744</v>
       </c>
     </row>
     <row r="137">
@@ -22618,13 +22618,13 @@
         <v>0.8</v>
       </c>
       <c r="Y138" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z138" t="b">
         <v>1</v>
       </c>
       <c r="AA138" t="n">
-        <v>0.7428516333872839</v>
+        <v>0.7432573286166072</v>
       </c>
     </row>
     <row r="139">
@@ -22792,13 +22792,13 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="Y140" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z140" t="b">
         <v>1</v>
       </c>
       <c r="AA140" t="n">
-        <v>0.5696714979963833</v>
+        <v>0.5699826139697908</v>
       </c>
     </row>
     <row r="141">
@@ -22966,13 +22966,13 @@
         <v>0.8620689655172414</v>
       </c>
       <c r="Y142" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z142" t="b">
         <v>1</v>
       </c>
       <c r="AA142" t="n">
-        <v>0.8004866739087111</v>
+        <v>0.8009238454920337</v>
       </c>
     </row>
     <row r="143">
@@ -23140,13 +23140,13 @@
         <v>0.28328611898017</v>
       </c>
       <c r="Y144" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z144" t="b">
         <v>1</v>
       </c>
       <c r="AA144" t="n">
-        <v>0.2630494452504546</v>
+        <v>0.2631931050342093</v>
       </c>
     </row>
     <row r="145">
@@ -23306,7 +23306,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr"/>
       <c r="Y146" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z146" t="b">
         <v>1</v>
@@ -23478,13 +23478,13 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="Y148" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z148" t="b">
         <v>1</v>
       </c>
       <c r="AA148" t="n">
-        <v>0.4380021423274079</v>
+        <v>0.4382413494201693</v>
       </c>
     </row>
     <row r="149">
@@ -23652,13 +23652,13 @@
         <v>0.2702702702702702</v>
       </c>
       <c r="Y150" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z150" t="b">
         <v>1</v>
       </c>
       <c r="AA150" t="n">
-        <v>0.2509633896578661</v>
+        <v>0.2511004488569619</v>
       </c>
     </row>
     <row r="151">
@@ -23826,13 +23826,13 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="Y152" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z152" t="b">
         <v>1</v>
       </c>
       <c r="AA152" t="n">
-        <v>0.383704356088473</v>
+        <v>0.3839139094094046</v>
       </c>
     </row>
     <row r="153">
@@ -23992,7 +23992,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr"/>
       <c r="Y154" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z154" t="b">
         <v>1</v>
@@ -24164,13 +24164,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y156" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z156" t="b">
         <v>1</v>
       </c>
       <c r="AA156" t="n">
-        <v>0.5216654728843285</v>
+        <v>0.5219503712195276</v>
       </c>
     </row>
     <row r="157">
@@ -24504,7 +24504,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr"/>
       <c r="Y160" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z160" t="b">
         <v>1</v>
@@ -24676,13 +24676,13 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="Y162" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z162" t="b">
         <v>1</v>
       </c>
       <c r="AA162" t="n">
-        <v>0.7549305217350445</v>
+        <v>0.7553428136347634</v>
       </c>
     </row>
     <row r="163">
@@ -24763,13 +24763,13 @@
         <v>0.2932551319648093</v>
       </c>
       <c r="Y163" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z163" t="b">
         <v>1</v>
       </c>
       <c r="AA163" t="n">
-        <v>0.2723063172240776</v>
+        <v>0.2724550324840935</v>
       </c>
     </row>
     <row r="164">
@@ -24850,13 +24850,13 @@
         <v>0.53475935828877</v>
       </c>
       <c r="Y164" t="n">
-        <v>0.07693106408358949</v>
+        <v>0.07634323833578012</v>
       </c>
       <c r="Z164" t="b">
         <v>1</v>
       </c>
       <c r="AA164" t="n">
-        <v>0.4965585784674356</v>
+        <v>0.4968297651180528</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update closing lines: Poll done: 24 snapshotted, 0 finalized with vig, 0 missed pre-match Wrote 91 matches to data/closing_lines/valorant_closing_lines.xlsx
</commit_message>
<xml_diff>
--- a/data/closing_lines/valorant_closing_lines.xlsx
+++ b/data/closing_lines/valorant_closing_lines.xlsx
@@ -756,7 +756,7 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
@@ -854,10 +854,10 @@
         <v>0.8</v>
       </c>
       <c r="V3" t="n">
-        <v>0.7432573286166072</v>
+        <v>0.7437374256440138</v>
       </c>
       <c r="W3" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X3" t="b">
         <v>1</v>
@@ -967,10 +967,10 @@
         <v>0.4901960784313725</v>
       </c>
       <c r="V4" t="n">
-        <v>0.4554272846915485</v>
+        <v>0.4557214617916751</v>
       </c>
       <c r="W4" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X4" t="b">
         <v>1</v>
@@ -1077,7 +1077,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
@@ -1187,10 +1187,10 @@
         <v>0.4975124378109453</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4622247068511239</v>
+        <v>0.4625232746542375</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X6" t="b">
         <v>1</v>
@@ -1389,10 +1389,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="V8" t="n">
-        <v>0.56307373380046</v>
+        <v>0.5634374436697074</v>
       </c>
       <c r="W8" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X8" t="b">
         <v>1</v>
@@ -1502,10 +1502,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="V9" t="n">
-        <v>0.7742263839756325</v>
+        <v>0.7747264850458477</v>
       </c>
       <c r="W9" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X9" t="b">
         <v>1</v>
@@ -1603,10 +1603,10 @@
         <v>0.6451612903225806</v>
       </c>
       <c r="V10" t="n">
-        <v>0.5994010714650058</v>
+        <v>0.5997882464871078</v>
       </c>
       <c r="W10" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X10" t="b">
         <v>1</v>
@@ -1716,10 +1716,10 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="V11" t="n">
-        <v>0.4576707688525907</v>
+        <v>0.4579663951009937</v>
       </c>
       <c r="W11" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
@@ -1829,10 +1829,10 @@
         <v>0.3802281368821293</v>
       </c>
       <c r="V12" t="n">
-        <v>0.3532591866048513</v>
+        <v>0.3534873696026682</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
@@ -2132,10 +2132,10 @@
         <v>0.6289308176100629</v>
       </c>
       <c r="V15" t="n">
-        <v>0.5843217992268924</v>
+        <v>0.5846992339968662</v>
       </c>
       <c r="W15" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X15" t="b">
         <v>1</v>
@@ -2346,10 +2346,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="V17" t="n">
-        <v>0.619381107180506</v>
+        <v>0.6197811880366781</v>
       </c>
       <c r="W17" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X17" t="b">
         <v>1</v>
@@ -2456,7 +2456,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
@@ -2566,10 +2566,10 @@
         <v>0.8928571428571428</v>
       </c>
       <c r="V19" t="n">
-        <v>0.8295282685453205</v>
+        <v>0.830064091120551</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X19" t="b">
         <v>1</v>
@@ -2679,10 +2679,10 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="V20" t="n">
-        <v>0.4321263538468647</v>
+        <v>0.4324054800255894</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
@@ -2792,10 +2792,10 @@
         <v>0.4566210045662101</v>
       </c>
       <c r="V21" t="n">
-        <v>0.4242336350551411</v>
+        <v>0.4245076630388207</v>
       </c>
       <c r="W21" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
@@ -2905,10 +2905,10 @@
         <v>0.4694835680751174</v>
       </c>
       <c r="V22" t="n">
-        <v>0.436183878296131</v>
+        <v>0.4364656253779424</v>
       </c>
       <c r="W22" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
@@ -3018,10 +3018,10 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="V23" t="n">
-        <v>0.5699826139697908</v>
+        <v>0.5703507865368204</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X23" t="b">
         <v>1</v>
@@ -3131,10 +3131,10 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="V24" t="n">
-        <v>0.5308980918690051</v>
+        <v>0.5312410183171526</v>
       </c>
       <c r="W24" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X24" t="b">
         <v>1</v>
@@ -3244,10 +3244,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="V25" t="n">
-        <v>0.7742263839756325</v>
+        <v>0.7747264850458477</v>
       </c>
       <c r="W25" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X25" t="b">
         <v>1</v>
@@ -3357,10 +3357,10 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="V26" t="n">
-        <v>0.4382413494201693</v>
+        <v>0.4385244254976496</v>
       </c>
       <c r="W26" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
@@ -3470,10 +3470,10 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="V27" t="n">
-        <v>0.645188653313027</v>
+        <v>0.645605404204873</v>
       </c>
       <c r="W27" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X27" t="b">
         <v>1</v>
@@ -3583,10 +3583,10 @@
         <v>0.3759398496240601</v>
       </c>
       <c r="V28" t="n">
-        <v>0.3492750604401349</v>
+        <v>0.3495006699454952</v>
       </c>
       <c r="W28" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X28" t="b">
         <v>1</v>
@@ -3696,10 +3696,10 @@
         <v>0.4629629629629629</v>
       </c>
       <c r="V29" t="n">
-        <v>0.4301257688753513</v>
+        <v>0.4304036028032487</v>
       </c>
       <c r="W29" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X29" t="b">
         <v>1</v>
@@ -3809,10 +3809,10 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="V30" t="n">
-        <v>0.6277511221424047</v>
+        <v>0.6281566094966332</v>
       </c>
       <c r="W30" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X30" t="b">
         <v>1</v>
@@ -3922,10 +3922,10 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="V31" t="n">
-        <v>0.491572307286116</v>
+        <v>0.4918898317751415</v>
       </c>
       <c r="W31" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X31" t="b">
         <v>1</v>
@@ -4032,7 +4032,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X32" t="b">
         <v>1</v>
@@ -4142,10 +4142,10 @@
         <v>0.8</v>
       </c>
       <c r="V33" t="n">
-        <v>0.7432573286166072</v>
+        <v>0.7437374256440138</v>
       </c>
       <c r="W33" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X33" t="b">
         <v>1</v>
@@ -4356,10 +4356,10 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="V35" t="n">
-        <v>0.3936744325299826</v>
+        <v>0.3939287212097531</v>
       </c>
       <c r="W35" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X35" t="b">
         <v>1</v>
@@ -4469,10 +4469,10 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="V36" t="n">
-        <v>0.5880200384625056</v>
+        <v>0.5883998620601374</v>
       </c>
       <c r="W36" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X36" t="b">
         <v>1</v>
@@ -4772,10 +4772,10 @@
         <v>0.591715976331361</v>
       </c>
       <c r="V39" t="n">
-        <v>0.5497465448347686</v>
+        <v>0.5501016461864008</v>
       </c>
       <c r="W39" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X39" t="b">
         <v>1</v>
@@ -4986,10 +4986,10 @@
         <v>0.8064516129032259</v>
       </c>
       <c r="V41" t="n">
-        <v>0.7492513393312573</v>
+        <v>0.7497353081088849</v>
       </c>
       <c r="W41" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X41" t="b">
         <v>1</v>
@@ -5096,7 +5096,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X42" t="b">
         <v>1</v>
@@ -5203,7 +5203,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X43" t="b">
         <v>1</v>
@@ -5310,7 +5310,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X44" t="b">
         <v>1</v>
@@ -5420,10 +5420,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="V45" t="n">
-        <v>0.619381107180506</v>
+        <v>0.6197811880366781</v>
       </c>
       <c r="W45" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X45" t="b">
         <v>1</v>
@@ -5533,10 +5533,10 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="V46" t="n">
-        <v>0.4424150765575042</v>
+        <v>0.4427008485976272</v>
       </c>
       <c r="W46" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X46" t="b">
         <v>1</v>
@@ -5646,10 +5646,10 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="V47" t="n">
-        <v>0.3936744325299826</v>
+        <v>0.3939287212097531</v>
       </c>
       <c r="W47" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X47" t="b">
         <v>1</v>
@@ -5759,10 +5759,10 @@
         <v>0.5</v>
       </c>
       <c r="V48" t="n">
-        <v>0.4645358303853795</v>
+        <v>0.4648358910275086</v>
       </c>
       <c r="W48" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X48" t="b">
         <v>1</v>
@@ -5869,7 +5869,7 @@
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X49" t="b">
         <v>1</v>
@@ -6080,10 +6080,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="V51" t="n">
-        <v>0.5219503712195276</v>
+        <v>0.5222875180084366</v>
       </c>
       <c r="W51" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X51" t="b">
         <v>1</v>
@@ -6193,10 +6193,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="V52" t="n">
-        <v>0.56307373380046</v>
+        <v>0.5634374436697074</v>
       </c>
       <c r="W52" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X52" t="b">
         <v>1</v>
@@ -6306,10 +6306,10 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="V53" t="n">
-        <v>0.5465127416298582</v>
+        <v>0.5468657541500102</v>
       </c>
       <c r="W53" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X53" t="b">
         <v>1</v>
@@ -6419,10 +6419,10 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="V54" t="n">
-        <v>0.6152792455435491</v>
+        <v>0.6156766768576274</v>
       </c>
       <c r="W54" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X54" t="b">
         <v>1</v>
@@ -6532,10 +6532,10 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="V55" t="n">
-        <v>0.5917653890259611</v>
+        <v>0.5921476318821766</v>
       </c>
       <c r="W55" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X55" t="b">
         <v>1</v>
@@ -6645,10 +6645,10 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="V56" t="n">
-        <v>0.4321263538468647</v>
+        <v>0.4324054800255894</v>
       </c>
       <c r="W56" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X56" t="b">
         <v>1</v>
@@ -6758,10 +6758,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="V57" t="n">
-        <v>0.6985501208802698</v>
+        <v>0.6990013398909903</v>
       </c>
       <c r="W57" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X57" t="b">
         <v>1</v>
@@ -6871,10 +6871,10 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="V58" t="n">
-        <v>0.4576707688525907</v>
+        <v>0.4579663951009937</v>
       </c>
       <c r="W58" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X58" t="b">
         <v>1</v>
@@ -6984,10 +6984,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="V59" t="n">
-        <v>0.5770631433358751</v>
+        <v>0.5774358894751659</v>
       </c>
       <c r="W59" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X59" t="b">
         <v>1</v>
@@ -7097,10 +7097,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="V60" t="n">
-        <v>0.6985501208802698</v>
+        <v>0.6990013398909903</v>
       </c>
       <c r="W60" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X60" t="b">
         <v>1</v>
@@ -7207,7 +7207,7 @@
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X61" t="b">
         <v>1</v>
@@ -7418,10 +7418,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="V63" t="n">
-        <v>0.3871131919878162</v>
+        <v>0.3873632425229239</v>
       </c>
       <c r="W63" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X63" t="b">
         <v>1</v>
@@ -7531,10 +7531,10 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="V64" t="n">
-        <v>0.6781544969129627</v>
+        <v>0.6785925416459979</v>
       </c>
       <c r="W64" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X64" t="b">
         <v>1</v>
@@ -7641,7 +7641,7 @@
       <c r="U65" t="inlineStr"/>
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X65" t="b">
         <v>1</v>
@@ -7751,10 +7751,10 @@
         <v>0.3521126760563381</v>
       </c>
       <c r="V66" t="n">
-        <v>0.3271379087220982</v>
+        <v>0.3273492190334568</v>
       </c>
       <c r="W66" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X66" t="b">
         <v>1</v>
@@ -7864,10 +7864,10 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="V67" t="n">
-        <v>0.6497004620774539</v>
+        <v>0.6501201273112009</v>
       </c>
       <c r="W67" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X67" t="b">
         <v>1</v>
@@ -7977,10 +7977,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="V68" t="n">
-        <v>0.5770631433358751</v>
+        <v>0.5774358894751659</v>
       </c>
       <c r="W68" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X68" t="b">
         <v>1</v>
@@ -8087,7 +8087,7 @@
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
       <c r="W69" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X69" t="b">
         <v>1</v>
@@ -8197,10 +8197,10 @@
         <v>0.8547008547008548</v>
       </c>
       <c r="V70" t="n">
-        <v>0.7940783425391102</v>
+        <v>0.79459126671369</v>
       </c>
       <c r="W70" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X70" t="b">
         <v>1</v>
@@ -8310,10 +8310,10 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="V71" t="n">
-        <v>0.6589160714686234</v>
+        <v>0.6593416894007215</v>
       </c>
       <c r="W71" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X71" t="b">
         <v>1</v>
@@ -8423,10 +8423,10 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="V72" t="n">
-        <v>0.7092150082219534</v>
+        <v>0.7096731160725321</v>
       </c>
       <c r="W72" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X72" t="b">
         <v>1</v>
@@ -8536,10 +8536,10 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="V73" t="n">
-        <v>0.559681723355879</v>
+        <v>0.5600432422018177</v>
       </c>
       <c r="W73" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X73" t="b">
         <v>1</v>
@@ -8649,10 +8649,10 @@
         <v>0.3731343283582089</v>
       </c>
       <c r="V74" t="n">
-        <v>0.3466685301383429</v>
+        <v>0.346892455990678</v>
       </c>
       <c r="W74" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X74" t="b">
         <v>1</v>
@@ -8762,10 +8762,10 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="V75" t="n">
-        <v>0.6497004620774539</v>
+        <v>0.6501201273112009</v>
       </c>
       <c r="W75" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X75" t="b">
         <v>1</v>
@@ -8875,10 +8875,10 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="V76" t="n">
-        <v>0.7202105897447744</v>
+        <v>0.720675800042649</v>
       </c>
       <c r="W76" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X76" t="b">
         <v>1</v>
@@ -8988,10 +8988,10 @@
         <v>0.8</v>
       </c>
       <c r="V77" t="n">
-        <v>0.7432573286166072</v>
+        <v>0.7437374256440138</v>
       </c>
       <c r="W77" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X77" t="b">
         <v>1</v>
@@ -9101,10 +9101,10 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="V78" t="n">
-        <v>0.5699826139697908</v>
+        <v>0.5703507865368204</v>
       </c>
       <c r="W78" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X78" t="b">
         <v>1</v>
@@ -9214,10 +9214,10 @@
         <v>0.8620689655172414</v>
       </c>
       <c r="V79" t="n">
-        <v>0.8009238454920337</v>
+        <v>0.8014411914267391</v>
       </c>
       <c r="W79" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X79" t="b">
         <v>1</v>
@@ -9327,10 +9327,10 @@
         <v>0.28328611898017</v>
       </c>
       <c r="V80" t="n">
-        <v>0.2631931050342093</v>
+        <v>0.2633631110637443</v>
       </c>
       <c r="W80" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X80" t="b">
         <v>1</v>
@@ -9437,7 +9437,7 @@
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr"/>
       <c r="W81" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X81" t="b">
         <v>1</v>
@@ -9547,10 +9547,10 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="V82" t="n">
-        <v>0.4382413494201693</v>
+        <v>0.4385244254976496</v>
       </c>
       <c r="W82" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X82" t="b">
         <v>1</v>
@@ -9660,10 +9660,10 @@
         <v>0.2702702702702702</v>
       </c>
       <c r="V83" t="n">
-        <v>0.2511004488569619</v>
+        <v>0.2512626437986533</v>
       </c>
       <c r="W83" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X83" t="b">
         <v>1</v>
@@ -9773,10 +9773,10 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="V84" t="n">
-        <v>0.3839139094094046</v>
+        <v>0.3841618934111641</v>
       </c>
       <c r="W84" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X84" t="b">
         <v>1</v>
@@ -9883,7 +9883,7 @@
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="inlineStr"/>
       <c r="W85" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X85" t="b">
         <v>1</v>
@@ -9993,10 +9993,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="V86" t="n">
-        <v>0.5219503712195276</v>
+        <v>0.5222875180084366</v>
       </c>
       <c r="W86" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X86" t="b">
         <v>1</v>
@@ -10305,7 +10305,7 @@
       <c r="U89" t="inlineStr"/>
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X89" t="b">
         <v>1</v>
@@ -10415,10 +10415,10 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="V90" t="n">
-        <v>0.7553428136347634</v>
+        <v>0.7558307171179002</v>
       </c>
       <c r="W90" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X90" t="b">
         <v>1</v>
@@ -10528,10 +10528,10 @@
         <v>0.2932551319648093</v>
       </c>
       <c r="V91" t="n">
-        <v>0.2724550324840935</v>
+        <v>0.2726310211305035</v>
       </c>
       <c r="W91" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X91" t="b">
         <v>1</v>
@@ -10629,10 +10629,10 @@
         <v>0.53475935828877</v>
       </c>
       <c r="V92" t="n">
-        <v>0.4968297651180528</v>
+        <v>0.4971506855909182</v>
       </c>
       <c r="W92" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="X92" t="b">
         <v>1</v>
@@ -10888,7 +10888,7 @@
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z2" t="b">
         <v>1</v>
@@ -11060,13 +11060,13 @@
         <v>0.8</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z4" t="b">
         <v>1</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.7432573286166072</v>
+        <v>0.7437374256440138</v>
       </c>
     </row>
     <row r="5">
@@ -11234,13 +11234,13 @@
         <v>0.4901960784313725</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z6" t="b">
         <v>1</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.4554272846915485</v>
+        <v>0.4557214617916751</v>
       </c>
     </row>
     <row r="7">
@@ -11400,7 +11400,7 @@
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z8" t="b">
         <v>1</v>
@@ -11485,13 +11485,13 @@
         <v>0.4975124378109453</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z9" t="b">
         <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.4622247068511239</v>
+        <v>0.4625232746542375</v>
       </c>
     </row>
     <row r="10">
@@ -11746,13 +11746,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z12" t="b">
         <v>1</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.56307373380046</v>
+        <v>0.5634374436697074</v>
       </c>
     </row>
     <row r="13">
@@ -11833,13 +11833,13 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z13" t="b">
         <v>1</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.7742263839756325</v>
+        <v>0.7747264850458477</v>
       </c>
     </row>
     <row r="14">
@@ -12007,13 +12007,13 @@
         <v>0.6451612903225806</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z15" t="b">
         <v>1</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.5994010714650058</v>
+        <v>0.5997882464871078</v>
       </c>
     </row>
     <row r="16">
@@ -12181,13 +12181,13 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z17" t="b">
         <v>1</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.4576707688525907</v>
+        <v>0.4579663951009937</v>
       </c>
     </row>
     <row r="18">
@@ -12268,13 +12268,13 @@
         <v>0.3802281368821293</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z18" t="b">
         <v>1</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.3532591866048513</v>
+        <v>0.3534873696026682</v>
       </c>
     </row>
     <row r="19">
@@ -12616,13 +12616,13 @@
         <v>0.6289308176100629</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z22" t="b">
         <v>1</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.5843217992268924</v>
+        <v>0.5846992339968662</v>
       </c>
     </row>
     <row r="23">
@@ -12877,13 +12877,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z25" t="b">
         <v>1</v>
       </c>
       <c r="AA25" t="n">
-        <v>0.619381107180506</v>
+        <v>0.6197811880366781</v>
       </c>
     </row>
     <row r="26">
@@ -13043,7 +13043,7 @@
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z27" t="b">
         <v>1</v>
@@ -13215,13 +13215,13 @@
         <v>0.8928571428571428</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z29" t="b">
         <v>1</v>
       </c>
       <c r="AA29" t="n">
-        <v>0.8295282685453205</v>
+        <v>0.830064091120551</v>
       </c>
     </row>
     <row r="30">
@@ -13389,13 +13389,13 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z31" t="b">
         <v>1</v>
       </c>
       <c r="AA31" t="n">
-        <v>0.4321263538468647</v>
+        <v>0.4324054800255894</v>
       </c>
     </row>
     <row r="32">
@@ -13563,13 +13563,13 @@
         <v>0.4566210045662101</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z33" t="b">
         <v>1</v>
       </c>
       <c r="AA33" t="n">
-        <v>0.4242336350551411</v>
+        <v>0.4245076630388207</v>
       </c>
     </row>
     <row r="34">
@@ -13737,13 +13737,13 @@
         <v>0.4694835680751174</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z35" t="b">
         <v>1</v>
       </c>
       <c r="AA35" t="n">
-        <v>0.436183878296131</v>
+        <v>0.4364656253779424</v>
       </c>
     </row>
     <row r="36">
@@ -13911,13 +13911,13 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z37" t="b">
         <v>1</v>
       </c>
       <c r="AA37" t="n">
-        <v>0.5699826139697908</v>
+        <v>0.5703507865368204</v>
       </c>
     </row>
     <row r="38">
@@ -14085,13 +14085,13 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z39" t="b">
         <v>1</v>
       </c>
       <c r="AA39" t="n">
-        <v>0.5308980918690051</v>
+        <v>0.5312410183171526</v>
       </c>
     </row>
     <row r="40">
@@ -14259,13 +14259,13 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z41" t="b">
         <v>1</v>
       </c>
       <c r="AA41" t="n">
-        <v>0.7742263839756325</v>
+        <v>0.7747264850458477</v>
       </c>
     </row>
     <row r="42">
@@ -14433,13 +14433,13 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z43" t="b">
         <v>1</v>
       </c>
       <c r="AA43" t="n">
-        <v>0.4382413494201693</v>
+        <v>0.4385244254976496</v>
       </c>
     </row>
     <row r="44">
@@ -14607,13 +14607,13 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z45" t="b">
         <v>1</v>
       </c>
       <c r="AA45" t="n">
-        <v>0.645188653313027</v>
+        <v>0.645605404204873</v>
       </c>
     </row>
     <row r="46">
@@ -14781,13 +14781,13 @@
         <v>0.3759398496240601</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z47" t="b">
         <v>1</v>
       </c>
       <c r="AA47" t="n">
-        <v>0.3492750604401349</v>
+        <v>0.3495006699454952</v>
       </c>
     </row>
     <row r="48">
@@ -14955,13 +14955,13 @@
         <v>0.4629629629629629</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z49" t="b">
         <v>1</v>
       </c>
       <c r="AA49" t="n">
-        <v>0.4301257688753513</v>
+        <v>0.4304036028032487</v>
       </c>
     </row>
     <row r="50">
@@ -15129,13 +15129,13 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z51" t="b">
         <v>1</v>
       </c>
       <c r="AA51" t="n">
-        <v>0.6277511221424047</v>
+        <v>0.6281566094966332</v>
       </c>
     </row>
     <row r="52">
@@ -15303,13 +15303,13 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z53" t="b">
         <v>1</v>
       </c>
       <c r="AA53" t="n">
-        <v>0.491572307286116</v>
+        <v>0.4918898317751415</v>
       </c>
     </row>
     <row r="54">
@@ -15469,7 +15469,7 @@
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr"/>
       <c r="Y55" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z55" t="b">
         <v>1</v>
@@ -15641,13 +15641,13 @@
         <v>0.8</v>
       </c>
       <c r="Y57" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z57" t="b">
         <v>1</v>
       </c>
       <c r="AA57" t="n">
-        <v>0.7432573286166072</v>
+        <v>0.7437374256440138</v>
       </c>
     </row>
     <row r="58">
@@ -15902,13 +15902,13 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="Y60" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z60" t="b">
         <v>1</v>
       </c>
       <c r="AA60" t="n">
-        <v>0.3936744325299826</v>
+        <v>0.3939287212097531</v>
       </c>
     </row>
     <row r="61">
@@ -15989,13 +15989,13 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z61" t="b">
         <v>1</v>
       </c>
       <c r="AA61" t="n">
-        <v>0.5880200384625056</v>
+        <v>0.5883998620601374</v>
       </c>
     </row>
     <row r="62">
@@ -16337,13 +16337,13 @@
         <v>0.591715976331361</v>
       </c>
       <c r="Y65" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z65" t="b">
         <v>1</v>
       </c>
       <c r="AA65" t="n">
-        <v>0.5497465448347686</v>
+        <v>0.5501016461864008</v>
       </c>
     </row>
     <row r="66">
@@ -16598,13 +16598,13 @@
         <v>0.8064516129032259</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z68" t="b">
         <v>1</v>
       </c>
       <c r="AA68" t="n">
-        <v>0.7492513393312573</v>
+        <v>0.7497353081088849</v>
       </c>
     </row>
     <row r="69">
@@ -16764,7 +16764,7 @@
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
       <c r="Y70" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z70" t="b">
         <v>1</v>
@@ -16928,7 +16928,7 @@
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr"/>
       <c r="Y72" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z72" t="b">
         <v>1</v>
@@ -17092,7 +17092,7 @@
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr"/>
       <c r="Y74" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z74" t="b">
         <v>1</v>
@@ -17264,13 +17264,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="Y76" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z76" t="b">
         <v>1</v>
       </c>
       <c r="AA76" t="n">
-        <v>0.619381107180506</v>
+        <v>0.6197811880366781</v>
       </c>
     </row>
     <row r="77">
@@ -17438,13 +17438,13 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="Y78" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z78" t="b">
         <v>1</v>
       </c>
       <c r="AA78" t="n">
-        <v>0.4424150765575042</v>
+        <v>0.4427008485976272</v>
       </c>
     </row>
     <row r="79">
@@ -17612,13 +17612,13 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z80" t="b">
         <v>1</v>
       </c>
       <c r="AA80" t="n">
-        <v>0.3936744325299826</v>
+        <v>0.3939287212097531</v>
       </c>
     </row>
     <row r="81">
@@ -17786,13 +17786,13 @@
         <v>0.5</v>
       </c>
       <c r="Y82" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z82" t="b">
         <v>1</v>
       </c>
       <c r="AA82" t="n">
-        <v>0.4645358303853795</v>
+        <v>0.4648358910275086</v>
       </c>
     </row>
     <row r="83">
@@ -17952,7 +17952,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr"/>
       <c r="Y84" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z84" t="b">
         <v>1</v>
@@ -18211,13 +18211,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y87" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z87" t="b">
         <v>1</v>
       </c>
       <c r="AA87" t="n">
-        <v>0.5219503712195276</v>
+        <v>0.5222875180084366</v>
       </c>
     </row>
     <row r="88">
@@ -18385,13 +18385,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z89" t="b">
         <v>1</v>
       </c>
       <c r="AA89" t="n">
-        <v>0.56307373380046</v>
+        <v>0.5634374436697074</v>
       </c>
     </row>
     <row r="90">
@@ -18559,13 +18559,13 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z91" t="b">
         <v>1</v>
       </c>
       <c r="AA91" t="n">
-        <v>0.5465127416298582</v>
+        <v>0.5468657541500102</v>
       </c>
     </row>
     <row r="92">
@@ -18733,13 +18733,13 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="Y93" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z93" t="b">
         <v>1</v>
       </c>
       <c r="AA93" t="n">
-        <v>0.6152792455435491</v>
+        <v>0.6156766768576274</v>
       </c>
     </row>
     <row r="94">
@@ -18907,13 +18907,13 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="Y95" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z95" t="b">
         <v>1</v>
       </c>
       <c r="AA95" t="n">
-        <v>0.5917653890259611</v>
+        <v>0.5921476318821766</v>
       </c>
     </row>
     <row r="96">
@@ -19081,13 +19081,13 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="Y97" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z97" t="b">
         <v>1</v>
       </c>
       <c r="AA97" t="n">
-        <v>0.4321263538468647</v>
+        <v>0.4324054800255894</v>
       </c>
     </row>
     <row r="98">
@@ -19255,13 +19255,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y99" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z99" t="b">
         <v>1</v>
       </c>
       <c r="AA99" t="n">
-        <v>0.6985501208802698</v>
+        <v>0.6990013398909903</v>
       </c>
     </row>
     <row r="100">
@@ -19429,13 +19429,13 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="Y101" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z101" t="b">
         <v>1</v>
       </c>
       <c r="AA101" t="n">
-        <v>0.4576707688525907</v>
+        <v>0.4579663951009937</v>
       </c>
     </row>
     <row r="102">
@@ -19603,13 +19603,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y103" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z103" t="b">
         <v>1</v>
       </c>
       <c r="AA103" t="n">
-        <v>0.5770631433358751</v>
+        <v>0.5774358894751659</v>
       </c>
     </row>
     <row r="104">
@@ -19777,13 +19777,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y105" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z105" t="b">
         <v>1</v>
       </c>
       <c r="AA105" t="n">
-        <v>0.6985501208802698</v>
+        <v>0.6990013398909903</v>
       </c>
     </row>
     <row r="106">
@@ -19943,7 +19943,7 @@
       <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr"/>
       <c r="Y107" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z107" t="b">
         <v>1</v>
@@ -20202,13 +20202,13 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="Y110" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z110" t="b">
         <v>1</v>
       </c>
       <c r="AA110" t="n">
-        <v>0.3871131919878162</v>
+        <v>0.3873632425229239</v>
       </c>
     </row>
     <row r="111">
@@ -20376,13 +20376,13 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="Y112" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z112" t="b">
         <v>1</v>
       </c>
       <c r="AA112" t="n">
-        <v>0.6781544969129627</v>
+        <v>0.6785925416459979</v>
       </c>
     </row>
     <row r="113">
@@ -20542,7 +20542,7 @@
       <c r="W114" t="inlineStr"/>
       <c r="X114" t="inlineStr"/>
       <c r="Y114" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z114" t="b">
         <v>1</v>
@@ -20714,13 +20714,13 @@
         <v>0.3521126760563381</v>
       </c>
       <c r="Y116" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z116" t="b">
         <v>1</v>
       </c>
       <c r="AA116" t="n">
-        <v>0.3271379087220982</v>
+        <v>0.3273492190334568</v>
       </c>
     </row>
     <row r="117">
@@ -20888,13 +20888,13 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="Y118" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z118" t="b">
         <v>1</v>
       </c>
       <c r="AA118" t="n">
-        <v>0.6497004620774539</v>
+        <v>0.6501201273112009</v>
       </c>
     </row>
     <row r="119">
@@ -21062,13 +21062,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y120" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z120" t="b">
         <v>1</v>
       </c>
       <c r="AA120" t="n">
-        <v>0.5770631433358751</v>
+        <v>0.5774358894751659</v>
       </c>
     </row>
     <row r="121">
@@ -21228,7 +21228,7 @@
       <c r="W122" t="inlineStr"/>
       <c r="X122" t="inlineStr"/>
       <c r="Y122" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z122" t="b">
         <v>1</v>
@@ -21400,13 +21400,13 @@
         <v>0.8547008547008548</v>
       </c>
       <c r="Y124" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z124" t="b">
         <v>1</v>
       </c>
       <c r="AA124" t="n">
-        <v>0.7940783425391102</v>
+        <v>0.79459126671369</v>
       </c>
     </row>
     <row r="125">
@@ -21574,13 +21574,13 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="Y126" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z126" t="b">
         <v>1</v>
       </c>
       <c r="AA126" t="n">
-        <v>0.6589160714686234</v>
+        <v>0.6593416894007215</v>
       </c>
     </row>
     <row r="127">
@@ -21748,13 +21748,13 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="Y128" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z128" t="b">
         <v>1</v>
       </c>
       <c r="AA128" t="n">
-        <v>0.7092150082219534</v>
+        <v>0.7096731160725321</v>
       </c>
     </row>
     <row r="129">
@@ -21922,13 +21922,13 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="Y130" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z130" t="b">
         <v>1</v>
       </c>
       <c r="AA130" t="n">
-        <v>0.559681723355879</v>
+        <v>0.5600432422018177</v>
       </c>
     </row>
     <row r="131">
@@ -22096,13 +22096,13 @@
         <v>0.3731343283582089</v>
       </c>
       <c r="Y132" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z132" t="b">
         <v>1</v>
       </c>
       <c r="AA132" t="n">
-        <v>0.3466685301383429</v>
+        <v>0.346892455990678</v>
       </c>
     </row>
     <row r="133">
@@ -22270,13 +22270,13 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="Y134" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z134" t="b">
         <v>1</v>
       </c>
       <c r="AA134" t="n">
-        <v>0.6497004620774539</v>
+        <v>0.6501201273112009</v>
       </c>
     </row>
     <row r="135">
@@ -22444,13 +22444,13 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="Y136" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z136" t="b">
         <v>1</v>
       </c>
       <c r="AA136" t="n">
-        <v>0.7202105897447744</v>
+        <v>0.720675800042649</v>
       </c>
     </row>
     <row r="137">
@@ -22618,13 +22618,13 @@
         <v>0.8</v>
       </c>
       <c r="Y138" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z138" t="b">
         <v>1</v>
       </c>
       <c r="AA138" t="n">
-        <v>0.7432573286166072</v>
+        <v>0.7437374256440138</v>
       </c>
     </row>
     <row r="139">
@@ -22792,13 +22792,13 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="Y140" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z140" t="b">
         <v>1</v>
       </c>
       <c r="AA140" t="n">
-        <v>0.5699826139697908</v>
+        <v>0.5703507865368204</v>
       </c>
     </row>
     <row r="141">
@@ -22966,13 +22966,13 @@
         <v>0.8620689655172414</v>
       </c>
       <c r="Y142" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z142" t="b">
         <v>1</v>
       </c>
       <c r="AA142" t="n">
-        <v>0.8009238454920337</v>
+        <v>0.8014411914267391</v>
       </c>
     </row>
     <row r="143">
@@ -23140,13 +23140,13 @@
         <v>0.28328611898017</v>
       </c>
       <c r="Y144" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z144" t="b">
         <v>1</v>
       </c>
       <c r="AA144" t="n">
-        <v>0.2631931050342093</v>
+        <v>0.2633631110637443</v>
       </c>
     </row>
     <row r="145">
@@ -23306,7 +23306,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr"/>
       <c r="Y146" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z146" t="b">
         <v>1</v>
@@ -23478,13 +23478,13 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="Y148" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z148" t="b">
         <v>1</v>
       </c>
       <c r="AA148" t="n">
-        <v>0.4382413494201693</v>
+        <v>0.4385244254976496</v>
       </c>
     </row>
     <row r="149">
@@ -23652,13 +23652,13 @@
         <v>0.2702702702702702</v>
       </c>
       <c r="Y150" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z150" t="b">
         <v>1</v>
       </c>
       <c r="AA150" t="n">
-        <v>0.2511004488569619</v>
+        <v>0.2512626437986533</v>
       </c>
     </row>
     <row r="151">
@@ -23826,13 +23826,13 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="Y152" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z152" t="b">
         <v>1</v>
       </c>
       <c r="AA152" t="n">
-        <v>0.3839139094094046</v>
+        <v>0.3841618934111641</v>
       </c>
     </row>
     <row r="153">
@@ -23992,7 +23992,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr"/>
       <c r="Y154" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z154" t="b">
         <v>1</v>
@@ -24164,13 +24164,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y156" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z156" t="b">
         <v>1</v>
       </c>
       <c r="AA156" t="n">
-        <v>0.5219503712195276</v>
+        <v>0.5222875180084366</v>
       </c>
     </row>
     <row r="157">
@@ -24504,7 +24504,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr"/>
       <c r="Y160" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z160" t="b">
         <v>1</v>
@@ -24676,13 +24676,13 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="Y162" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z162" t="b">
         <v>1</v>
       </c>
       <c r="AA162" t="n">
-        <v>0.7553428136347634</v>
+        <v>0.7558307171179002</v>
       </c>
     </row>
     <row r="163">
@@ -24763,13 +24763,13 @@
         <v>0.2932551319648093</v>
       </c>
       <c r="Y163" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z163" t="b">
         <v>1</v>
       </c>
       <c r="AA163" t="n">
-        <v>0.2724550324840935</v>
+        <v>0.2726310211305035</v>
       </c>
     </row>
     <row r="164">
@@ -24850,13 +24850,13 @@
         <v>0.53475935828877</v>
       </c>
       <c r="Y164" t="n">
-        <v>0.07634323833578012</v>
+        <v>0.07564843776318994</v>
       </c>
       <c r="Z164" t="b">
         <v>1</v>
       </c>
       <c r="AA164" t="n">
-        <v>0.4968297651180528</v>
+        <v>0.4971506855909182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update closing lines: Poll done: 23 snapshotted, 0 finalized with vig, 0 missed pre-match Wrote 93 matches to data/closing_lines/valorant_closing_lines.xlsx
</commit_message>
<xml_diff>
--- a/data/closing_lines/valorant_closing_lines.xlsx
+++ b/data/closing_lines/valorant_closing_lines.xlsx
@@ -998,7 +998,7 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X4" t="b">
         <v>1</v>
@@ -1096,10 +1096,10 @@
         <v>0.8</v>
       </c>
       <c r="V5" t="n">
-        <v>0.7424113926068979</v>
+        <v>0.7440116849044103</v>
       </c>
       <c r="W5" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
@@ -1122,10 +1122,10 @@
         <v>0.819672131147541</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.7694871792661078</v>
+        <v>0.7706180549689851</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL5" t="b">
         <v>1</v>
@@ -1209,10 +1209,10 @@
         <v>0.4901960784313725</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4549089415483443</v>
+        <v>0.4558895128090749</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X6" t="b">
         <v>1</v>
@@ -1235,10 +1235,10 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.496706009896641</v>
+        <v>0.497435993154583</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL6" t="b">
         <v>1</v>
@@ -1319,7 +1319,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X7" t="b">
         <v>1</v>
@@ -1342,10 +1342,10 @@
         <v>0.4464285714285714</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.4190956958502908</v>
+        <v>0.4197116192241793</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL7" t="b">
         <v>1</v>
@@ -1429,10 +1429,10 @@
         <v>0.4975124378109453</v>
       </c>
       <c r="V8" t="n">
-        <v>0.4616986272430957</v>
+        <v>0.4626938338957776</v>
       </c>
       <c r="W8" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X8" t="b">
         <v>1</v>
@@ -1544,10 +1544,10 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.6852367581785777</v>
+        <v>0.6862438153738407</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL9" t="b">
         <v>1</v>
@@ -1631,10 +1631,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="V10" t="n">
-        <v>0.5624328731870438</v>
+        <v>0.5636452158366745</v>
       </c>
       <c r="W10" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X10" t="b">
         <v>1</v>
@@ -1657,10 +1657,10 @@
         <v>0.5464480874316939</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.5129914528440718</v>
+        <v>0.5137453699793233</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL10" t="b">
         <v>1</v>
@@ -1744,10 +1744,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="V11" t="n">
-        <v>0.7733452006321854</v>
+        <v>0.7750121717754274</v>
       </c>
       <c r="W11" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
@@ -1845,10 +1845,10 @@
         <v>0.6451612903225806</v>
       </c>
       <c r="V12" t="n">
-        <v>0.5987188650055628</v>
+        <v>0.6000094233100083</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
@@ -1871,10 +1871,10 @@
         <v>0.5952380952380952</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.5587942611337211</v>
+        <v>0.5596154922989058</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL12" t="b">
         <v>1</v>
@@ -1958,10 +1958,10 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="V13" t="n">
-        <v>0.4571498722948879</v>
+        <v>0.4581352739559177</v>
       </c>
       <c r="W13" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
@@ -1984,10 +1984,10 @@
         <v>0.5681818181818182</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.5333945219912792</v>
+        <v>0.5341784244671374</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL13" t="b">
         <v>1</v>
@@ -2071,10 +2071,10 @@
         <v>0.3802281368821293</v>
       </c>
       <c r="V14" t="n">
-        <v>0.3528571257637347</v>
+        <v>0.3536177209621722</v>
       </c>
       <c r="W14" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
@@ -2186,10 +2186,10 @@
         <v>0.4065040650406504</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.3816155929693705</v>
+        <v>0.3821764337651064</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL15" t="b">
         <v>1</v>
@@ -2287,10 +2287,10 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.7277320610113577</v>
+        <v>0.7288015713660168</v>
       </c>
       <c r="AK16" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL16" t="b">
         <v>1</v>
@@ -2374,10 +2374,10 @@
         <v>0.6289308176100629</v>
       </c>
       <c r="V17" t="n">
-        <v>0.5836567551941021</v>
+        <v>0.584914846622964</v>
       </c>
       <c r="W17" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X17" t="b">
         <v>1</v>
@@ -2400,10 +2400,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.5689541567906978</v>
+        <v>0.5697903194316132</v>
       </c>
       <c r="AK17" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL17" t="b">
         <v>1</v>
@@ -2501,10 +2501,10 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0.4470354089069768</v>
+        <v>0.4476923938391246</v>
       </c>
       <c r="AK18" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL18" t="b">
         <v>1</v>
@@ -2588,10 +2588,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="V19" t="n">
-        <v>0.6186761605057483</v>
+        <v>0.6200097374203418</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X19" t="b">
         <v>1</v>
@@ -2614,10 +2614,10 @@
         <v>0.6578947368421053</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.6176147096741128</v>
+        <v>0.6185223862251065</v>
       </c>
       <c r="AK19" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL19" t="b">
         <v>1</v>
@@ -2698,7 +2698,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
@@ -2721,10 +2721,10 @@
         <v>0.3571428571428572</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0.3352765566802327</v>
+        <v>0.3357692953793435</v>
       </c>
       <c r="AK20" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL20" t="b">
         <v>1</v>
@@ -2808,10 +2808,10 @@
         <v>0.8928571428571428</v>
       </c>
       <c r="V21" t="n">
-        <v>0.8285841435344842</v>
+        <v>0.8303701840451007</v>
       </c>
       <c r="W21" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
@@ -2834,10 +2834,10 @@
         <v>0.9174311926605504</v>
       </c>
       <c r="AJ21" t="n">
-        <v>0.8612608795455517</v>
+        <v>0.8625266303322584</v>
       </c>
       <c r="AK21" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL21" t="b">
         <v>1</v>
@@ -2921,10 +2921,10 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="V22" t="n">
-        <v>0.4316345305854057</v>
+        <v>0.4325649330839594</v>
       </c>
       <c r="W22" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
@@ -2947,10 +2947,10 @@
         <v>0.4273504273504274</v>
       </c>
       <c r="AJ22" t="n">
-        <v>0.4011856233780562</v>
+        <v>0.4017752252402401</v>
       </c>
       <c r="AK22" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL22" t="b">
         <v>1</v>
@@ -3034,10 +3034,10 @@
         <v>0.4566210045662101</v>
       </c>
       <c r="V23" t="n">
-        <v>0.4237507948669509</v>
+        <v>0.424664203712563</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X23" t="b">
         <v>1</v>
@@ -3060,10 +3060,10 @@
         <v>0.4587155963302752</v>
       </c>
       <c r="AJ23" t="n">
-        <v>0.4306304397727759</v>
+        <v>0.4312633151661292</v>
       </c>
       <c r="AK23" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL23" t="b">
         <v>1</v>
@@ -3147,10 +3147,10 @@
         <v>0.4694835680751174</v>
       </c>
       <c r="V24" t="n">
-        <v>0.435687436975879</v>
+        <v>0.4366265756481281</v>
       </c>
       <c r="W24" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X24" t="b">
         <v>1</v>
@@ -3173,10 +3173,10 @@
         <v>0.495049504950495</v>
       </c>
       <c r="AJ24" t="n">
-        <v>0.4647397815369562</v>
+        <v>0.4654227856743375</v>
       </c>
       <c r="AK24" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL24" t="b">
         <v>1</v>
@@ -3260,10 +3260,10 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="V25" t="n">
-        <v>0.5693338900359647</v>
+        <v>0.5705611080555294</v>
       </c>
       <c r="W25" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X25" t="b">
         <v>1</v>
@@ -3286,10 +3286,10 @@
         <v>0.625</v>
       </c>
       <c r="AJ25" t="n">
-        <v>0.5867339741904072</v>
+        <v>0.5875962669138511</v>
       </c>
       <c r="AK25" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL25" t="b">
         <v>1</v>
@@ -3373,10 +3373,10 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="V26" t="n">
-        <v>0.5302938518620699</v>
+        <v>0.5314369177888645</v>
       </c>
       <c r="W26" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
@@ -3399,10 +3399,10 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="AJ26" t="n">
-        <v>0.5655267221112359</v>
+        <v>0.5663578476278083</v>
       </c>
       <c r="AK26" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL26" t="b">
         <v>1</v>
@@ -3486,10 +3486,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="V27" t="n">
-        <v>0.7733452006321854</v>
+        <v>0.7750121717754274</v>
       </c>
       <c r="W27" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X27" t="b">
         <v>1</v>
@@ -3512,10 +3512,10 @@
         <v>0.8474576271186441</v>
       </c>
       <c r="AJ27" t="n">
-        <v>0.7955714904276707</v>
+        <v>0.7967407009001372</v>
       </c>
       <c r="AK27" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL27" t="b">
         <v>1</v>
@@ -3599,10 +3599,10 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="V28" t="n">
-        <v>0.4377425663955765</v>
+        <v>0.438686134967223</v>
       </c>
       <c r="W28" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X28" t="b">
         <v>1</v>
@@ -3625,10 +3625,10 @@
         <v>0.4545454545454545</v>
       </c>
       <c r="AJ28" t="n">
-        <v>0.4267156175930233</v>
+        <v>0.4273427395737099</v>
       </c>
       <c r="AK28" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL28" t="b">
         <v>1</v>
@@ -3712,10 +3712,10 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="V29" t="n">
-        <v>0.6444543338601544</v>
+        <v>0.6458434764795228</v>
       </c>
       <c r="W29" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X29" t="b">
         <v>1</v>
@@ -3738,10 +3738,10 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="AJ29" t="n">
-        <v>0.6657974175210294</v>
+        <v>0.6667759057178453</v>
       </c>
       <c r="AK29" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL29" t="b">
         <v>1</v>
@@ -3825,10 +3825,10 @@
         <v>0.3759398496240601</v>
       </c>
       <c r="V30" t="n">
-        <v>0.3488775341197828</v>
+        <v>0.3496295511768845</v>
       </c>
       <c r="W30" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X30" t="b">
         <v>1</v>
@@ -3851,10 +3851,10 @@
         <v>0.3968253968253968</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.3725295074224807</v>
+        <v>0.3730769948659372</v>
       </c>
       <c r="AK30" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL30" t="b">
         <v>1</v>
@@ -3938,10 +3938,10 @@
         <v>0.4629629629629629</v>
       </c>
       <c r="V31" t="n">
-        <v>0.4296362225734362</v>
+        <v>0.4305623176530151</v>
       </c>
       <c r="W31" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X31" t="b">
         <v>1</v>
@@ -3964,10 +3964,10 @@
         <v>0.4672897196261682</v>
       </c>
       <c r="AJ31" t="n">
-        <v>0.4386796068713325</v>
+        <v>0.4393243117112905</v>
       </c>
       <c r="AK31" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL31" t="b">
         <v>1</v>
@@ -4051,10 +4051,10 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="V32" t="n">
-        <v>0.6270366491612313</v>
+        <v>0.6283882473854816</v>
       </c>
       <c r="W32" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X32" t="b">
         <v>1</v>
@@ -4077,10 +4077,10 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="AJ32" t="n">
-        <v>0.6217048733143388</v>
+        <v>0.6226185609683191</v>
       </c>
       <c r="AK32" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL32" t="b">
         <v>1</v>
@@ -4164,10 +4164,10 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="V33" t="n">
-        <v>0.491012825798213</v>
+        <v>0.4920712201748746</v>
       </c>
       <c r="W33" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X33" t="b">
         <v>1</v>
@@ -4190,10 +4190,10 @@
         <v>0.5319148936170213</v>
       </c>
       <c r="AJ33" t="n">
-        <v>0.499348063140772</v>
+        <v>0.5000819292883839</v>
       </c>
       <c r="AK33" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL33" t="b">
         <v>1</v>
@@ -4274,7 +4274,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X34" t="b">
         <v>1</v>
@@ -4297,10 +4297,10 @@
         <v>0.8264462809917356</v>
       </c>
       <c r="AJ34" t="n">
-        <v>0.7758465774418607</v>
+        <v>0.7769867992249271</v>
       </c>
       <c r="AK34" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL34" t="b">
         <v>1</v>
@@ -4384,10 +4384,10 @@
         <v>0.8</v>
       </c>
       <c r="V35" t="n">
-        <v>0.7424113926068979</v>
+        <v>0.7440116849044103</v>
       </c>
       <c r="W35" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X35" t="b">
         <v>1</v>
@@ -4410,10 +4410,10 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="AJ35" t="n">
-        <v>0.763231185938741</v>
+        <v>0.7643528675302128</v>
       </c>
       <c r="AK35" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL35" t="b">
         <v>1</v>
@@ -4511,10 +4511,10 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="AJ36" t="n">
-        <v>0.6343069991247645</v>
+        <v>0.6352392074744336</v>
       </c>
       <c r="AK36" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL36" t="b">
         <v>1</v>
@@ -4598,10 +4598,10 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="V37" t="n">
-        <v>0.3932263732028061</v>
+        <v>0.3940739856485224</v>
       </c>
       <c r="W37" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X37" t="b">
         <v>1</v>
@@ -4624,10 +4624,10 @@
         <v>0.4347826086956522</v>
       </c>
       <c r="AJ37" t="n">
-        <v>0.4081627646541963</v>
+        <v>0.4087626204618095</v>
       </c>
       <c r="AK37" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL37" t="b">
         <v>1</v>
@@ -4711,10 +4711,10 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="V38" t="n">
-        <v>0.5873507852902673</v>
+        <v>0.5886168393231093</v>
       </c>
       <c r="W38" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X38" t="b">
         <v>1</v>
@@ -4826,10 +4826,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="AJ39" t="n">
-        <v>0.7058453824847003</v>
+        <v>0.7068827271144072</v>
       </c>
       <c r="AK39" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL39" t="b">
         <v>1</v>
@@ -4927,10 +4927,10 @@
         <v>0.9345794392523364</v>
       </c>
       <c r="AJ40" t="n">
-        <v>0.8773592137426649</v>
+        <v>0.8786486234225811</v>
       </c>
       <c r="AK40" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL40" t="b">
         <v>1</v>
@@ -5014,10 +5014,10 @@
         <v>0.591715976331361</v>
       </c>
       <c r="V41" t="n">
-        <v>0.549120852519895</v>
+        <v>0.5503045006689425</v>
       </c>
       <c r="W41" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X41" t="b">
         <v>1</v>
@@ -5040,10 +5040,10 @@
         <v>0.6097560975609756</v>
       </c>
       <c r="AJ41" t="n">
-        <v>0.5724233894540557</v>
+        <v>0.5732646506476596</v>
       </c>
       <c r="AK41" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL41" t="b">
         <v>1</v>
@@ -5141,10 +5141,10 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="AJ42" t="n">
-        <v>0.763231185938741</v>
+        <v>0.7643528675302128</v>
       </c>
       <c r="AK42" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL42" t="b">
         <v>1</v>
@@ -5228,10 +5228,10 @@
         <v>0.8064516129032259</v>
       </c>
       <c r="V43" t="n">
-        <v>0.7483985812569536</v>
+        <v>0.7500117791375104</v>
       </c>
       <c r="W43" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X43" t="b">
         <v>1</v>
@@ -5254,10 +5254,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="AJ43" t="n">
-        <v>0.7058453824847003</v>
+        <v>0.7068827271144072</v>
       </c>
       <c r="AK43" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL43" t="b">
         <v>1</v>
@@ -5338,7 +5338,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X44" t="b">
         <v>1</v>
@@ -5361,10 +5361,10 @@
         <v>0.8</v>
       </c>
       <c r="AJ44" t="n">
-        <v>0.7510194869637212</v>
+        <v>0.7521232216497294</v>
       </c>
       <c r="AK44" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL44" t="b">
         <v>1</v>
@@ -5445,7 +5445,7 @@
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X45" t="b">
         <v>1</v>
@@ -5468,10 +5468,10 @@
         <v>0.8264462809917356</v>
       </c>
       <c r="AJ45" t="n">
-        <v>0.7758465774418607</v>
+        <v>0.7769867992249271</v>
       </c>
       <c r="AK45" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL45" t="b">
         <v>1</v>
@@ -5552,7 +5552,7 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X46" t="b">
         <v>1</v>
@@ -5575,10 +5575,10 @@
         <v>0.8403361344537815</v>
       </c>
       <c r="AJ46" t="n">
-        <v>0.7888860157181945</v>
+        <v>0.7900454008925729</v>
       </c>
       <c r="AK46" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL46" t="b">
         <v>1</v>
@@ -5662,10 +5662,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="V47" t="n">
-        <v>0.6186761605057483</v>
+        <v>0.6200097374203418</v>
       </c>
       <c r="W47" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X47" t="b">
         <v>1</v>
@@ -5688,10 +5688,10 @@
         <v>0.591715976331361</v>
       </c>
       <c r="AJ47" t="n">
-        <v>0.5554877862157701</v>
+        <v>0.5563041580249478</v>
       </c>
       <c r="AK47" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL47" t="b">
         <v>1</v>
@@ -5775,10 +5775,10 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="V48" t="n">
-        <v>0.4419115432183915</v>
+        <v>0.442864098157387</v>
       </c>
       <c r="W48" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X48" t="b">
         <v>1</v>
@@ -5801,10 +5801,10 @@
         <v>0.4464285714285714</v>
       </c>
       <c r="AJ48" t="n">
-        <v>0.4190956958502908</v>
+        <v>0.4197116192241793</v>
       </c>
       <c r="AK48" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL48" t="b">
         <v>1</v>
@@ -5888,10 +5888,10 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="V49" t="n">
-        <v>0.3932263732028061</v>
+        <v>0.3940739856485224</v>
       </c>
       <c r="W49" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X49" t="b">
         <v>1</v>
@@ -5914,10 +5914,10 @@
         <v>0.4065040650406504</v>
       </c>
       <c r="AJ49" t="n">
-        <v>0.3816155929693705</v>
+        <v>0.3821764337651064</v>
       </c>
       <c r="AK49" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL49" t="b">
         <v>1</v>
@@ -6001,10 +6001,10 @@
         <v>0.5</v>
       </c>
       <c r="V50" t="n">
-        <v>0.4640071203793112</v>
+        <v>0.4650073030652564</v>
       </c>
       <c r="W50" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X50" t="b">
         <v>1</v>
@@ -6027,10 +6027,10 @@
         <v>0.5102040816326531</v>
       </c>
       <c r="AJ50" t="n">
-        <v>0.4789665095431895</v>
+        <v>0.4796704219704907</v>
       </c>
       <c r="AK50" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL50" t="b">
         <v>1</v>
@@ -6111,7 +6111,7 @@
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr"/>
       <c r="W51" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X51" t="b">
         <v>1</v>
@@ -6134,10 +6134,10 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="AJ51" t="n">
-        <v>0.5522202110027361</v>
+        <v>0.5530317806248011</v>
       </c>
       <c r="AK51" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL51" t="b">
         <v>1</v>
@@ -6235,10 +6235,10 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="AJ52" t="n">
-        <v>0.7277320610113577</v>
+        <v>0.7288015713660168</v>
       </c>
       <c r="AK52" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL52" t="b">
         <v>1</v>
@@ -6322,10 +6322,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="V53" t="n">
-        <v>0.5213563150329339</v>
+        <v>0.5224801158036589</v>
       </c>
       <c r="W53" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X53" t="b">
         <v>1</v>
@@ -6348,10 +6348,10 @@
         <v>0.5494505494505494</v>
       </c>
       <c r="AJ53" t="n">
-        <v>0.5158100872003578</v>
+        <v>0.5165681467374514</v>
       </c>
       <c r="AK53" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL53" t="b">
         <v>1</v>
@@ -6435,10 +6435,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="V54" t="n">
-        <v>0.5624328731870438</v>
+        <v>0.5636452158366745</v>
       </c>
       <c r="W54" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X54" t="b">
         <v>1</v>
@@ -6461,10 +6461,10 @@
         <v>0.5988023952095809</v>
       </c>
       <c r="AJ54" t="n">
-        <v>0.5621403345536835</v>
+        <v>0.5629664832707556</v>
       </c>
       <c r="AK54" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL54" t="b">
         <v>1</v>
@@ -6548,10 +6548,10 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="V55" t="n">
-        <v>0.5458907298580131</v>
+        <v>0.5470674153708899</v>
       </c>
       <c r="W55" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X55" t="b">
         <v>1</v>
@@ -6574,10 +6574,10 @@
         <v>0.5988023952095809</v>
       </c>
       <c r="AJ55" t="n">
-        <v>0.5621403345536835</v>
+        <v>0.5629664832707556</v>
       </c>
       <c r="AK55" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL55" t="b">
         <v>1</v>
@@ -6661,10 +6661,10 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="V56" t="n">
-        <v>0.6145789673898162</v>
+        <v>0.6159037126692138</v>
       </c>
       <c r="W56" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X56" t="b">
         <v>1</v>
@@ -6687,10 +6687,10 @@
         <v>0.6578947368421053</v>
       </c>
       <c r="AJ56" t="n">
-        <v>0.6176147096741128</v>
+        <v>0.6185223862251065</v>
       </c>
       <c r="AK56" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL56" t="b">
         <v>1</v>
@@ -6774,10 +6774,10 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="V57" t="n">
-        <v>0.5910918730946639</v>
+        <v>0.5923659911659317</v>
       </c>
       <c r="W57" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X57" t="b">
         <v>1</v>
@@ -6800,10 +6800,10 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="AJ57" t="n">
-        <v>0.5941609865219312</v>
+        <v>0.5950341943431403</v>
       </c>
       <c r="AK57" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL57" t="b">
         <v>1</v>
@@ -6887,10 +6887,10 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="V58" t="n">
-        <v>0.4316345305854057</v>
+        <v>0.4325649330839594</v>
       </c>
       <c r="W58" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X58" t="b">
         <v>1</v>
@@ -6913,10 +6913,10 @@
         <v>0.4672897196261682</v>
       </c>
       <c r="AJ58" t="n">
-        <v>0.4386796068713325</v>
+        <v>0.4393243117112905</v>
       </c>
       <c r="AK58" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL58" t="b">
         <v>1</v>
@@ -7000,10 +7000,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="V59" t="n">
-        <v>0.6977550682395657</v>
+        <v>0.699259102353769</v>
       </c>
       <c r="W59" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X59" t="b">
         <v>1</v>
@@ -7026,10 +7026,10 @@
         <v>0.7692307692307692</v>
       </c>
       <c r="AJ59" t="n">
-        <v>0.722134122080501</v>
+        <v>0.723195405432432</v>
       </c>
       <c r="AK59" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL59" t="b">
         <v>1</v>
@@ -7113,10 +7113,10 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="V60" t="n">
-        <v>0.4571498722948879</v>
+        <v>0.4581352739559177</v>
       </c>
       <c r="W60" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X60" t="b">
         <v>1</v>
@@ -7139,10 +7139,10 @@
         <v>0.495049504950495</v>
       </c>
       <c r="AJ60" t="n">
-        <v>0.4647397815369562</v>
+        <v>0.4654227856743375</v>
       </c>
       <c r="AK60" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL60" t="b">
         <v>1</v>
@@ -7226,10 +7226,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="V61" t="n">
-        <v>0.5764063607196411</v>
+        <v>0.5776488236835483</v>
       </c>
       <c r="W61" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X61" t="b">
         <v>1</v>
@@ -7252,10 +7252,10 @@
         <v>0.6097560975609756</v>
       </c>
       <c r="AJ61" t="n">
-        <v>0.5724233894540557</v>
+        <v>0.5732646506476596</v>
       </c>
       <c r="AK61" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL61" t="b">
         <v>1</v>
@@ -7339,10 +7339,10 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="V62" t="n">
-        <v>0.6977550682395657</v>
+        <v>0.699259102353769</v>
       </c>
       <c r="W62" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X62" t="b">
         <v>1</v>
@@ -7365,10 +7365,10 @@
         <v>0.7692307692307692</v>
       </c>
       <c r="AJ62" t="n">
-        <v>0.722134122080501</v>
+        <v>0.723195405432432</v>
       </c>
       <c r="AK62" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL62" t="b">
         <v>1</v>
@@ -7449,7 +7449,7 @@
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr"/>
       <c r="W63" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X63" t="b">
         <v>1</v>
@@ -7472,10 +7472,10 @@
         <v>0.3472222222222222</v>
       </c>
       <c r="AJ63" t="n">
-        <v>0.3259633189946706</v>
+        <v>0.326442370507695</v>
       </c>
       <c r="AK63" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL63" t="b">
         <v>1</v>
@@ -7573,10 +7573,10 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="AJ64" t="n">
-        <v>0.5689541567906978</v>
+        <v>0.5697903194316132</v>
       </c>
       <c r="AK64" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL64" t="b">
         <v>1</v>
@@ -7660,10 +7660,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="V65" t="n">
-        <v>0.3866726003160927</v>
+        <v>0.3875060858877137</v>
       </c>
       <c r="W65" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X65" t="b">
         <v>1</v>
@@ -7686,10 +7686,10 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="AJ65" t="n">
-        <v>0.3879232887209303</v>
+        <v>0.3884933996124635</v>
       </c>
       <c r="AK65" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL65" t="b">
         <v>1</v>
@@ -7773,10 +7773,10 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="V66" t="n">
-        <v>0.6773826574880455</v>
+        <v>0.6788427781974546</v>
       </c>
       <c r="W66" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X66" t="b">
         <v>1</v>
@@ -7799,10 +7799,10 @@
         <v>0.7407407407407407</v>
       </c>
       <c r="AJ66" t="n">
-        <v>0.6953884138552974</v>
+        <v>0.6964103904164161</v>
       </c>
       <c r="AK66" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL66" t="b">
         <v>1</v>
@@ -7883,7 +7883,7 @@
       <c r="U67" t="inlineStr"/>
       <c r="V67" t="inlineStr"/>
       <c r="W67" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X67" t="b">
         <v>1</v>
@@ -7906,10 +7906,10 @@
         <v>0.8849557522123894</v>
       </c>
       <c r="AJ67" t="n">
-        <v>0.8307737687651783</v>
+        <v>0.8319947142143025</v>
       </c>
       <c r="AK67" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL67" t="b">
         <v>1</v>
@@ -7993,10 +7993,10 @@
         <v>0.3521126760563381</v>
       </c>
       <c r="V68" t="n">
-        <v>0.3267655777319093</v>
+        <v>0.3274699317360961</v>
       </c>
       <c r="W68" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X68" t="b">
         <v>1</v>
@@ -8019,10 +8019,10 @@
         <v>0.3378378378378378</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.3171534995623823</v>
+        <v>0.3176196037372168</v>
       </c>
       <c r="AK68" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL68" t="b">
         <v>1</v>
@@ -8106,10 +8106,10 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="V69" t="n">
-        <v>0.6489610075235122</v>
+        <v>0.6503598644269322</v>
       </c>
       <c r="W69" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X69" t="b">
         <v>1</v>
@@ -8132,10 +8132,10 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="AJ69" t="n">
-        <v>0.6657974175210294</v>
+        <v>0.6667759057178453</v>
       </c>
       <c r="AK69" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL69" t="b">
         <v>1</v>
@@ -8219,10 +8219,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="V70" t="n">
-        <v>0.5764063607196411</v>
+        <v>0.5776488236835483</v>
       </c>
       <c r="W70" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X70" t="b">
         <v>1</v>
@@ -8245,10 +8245,10 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="AJ70" t="n">
-        <v>0.5979454514042366</v>
+        <v>0.5988242210587017</v>
       </c>
       <c r="AK70" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL70" t="b">
         <v>1</v>
@@ -8329,7 +8329,7 @@
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X71" t="b">
         <v>1</v>
@@ -8352,10 +8352,10 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="AJ71" t="n">
-        <v>0.6519266379893413</v>
+        <v>0.6528847410153901</v>
       </c>
       <c r="AK71" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL71" t="b">
         <v>1</v>
@@ -8439,10 +8439,10 @@
         <v>0.8547008547008548</v>
       </c>
       <c r="V72" t="n">
-        <v>0.7931745647509594</v>
+        <v>0.7948842787440281</v>
       </c>
       <c r="W72" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X72" t="b">
         <v>1</v>
@@ -8465,10 +8465,10 @@
         <v>0.8771929824561404</v>
       </c>
       <c r="AJ72" t="n">
-        <v>0.8234862795654838</v>
+        <v>0.8246965149668086</v>
       </c>
       <c r="AK72" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL72" t="b">
         <v>1</v>
@@ -8552,10 +8552,10 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="V73" t="n">
-        <v>0.6581661281976046</v>
+        <v>0.6595848270429169</v>
       </c>
       <c r="W73" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X73" t="b">
         <v>1</v>
@@ -8578,10 +8578,10 @@
         <v>0.7042253521126761</v>
       </c>
       <c r="AJ73" t="n">
-        <v>0.6611087033131349</v>
+        <v>0.6620803007480013</v>
       </c>
       <c r="AK73" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL73" t="b">
         <v>1</v>
@@ -8665,10 +8665,10 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="V74" t="n">
-        <v>0.7084078173729941</v>
+        <v>0.7099348138400861</v>
       </c>
       <c r="W74" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X74" t="b">
         <v>1</v>
@@ -8691,10 +8691,10 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="AJ74" t="n">
-        <v>0.7166216478661461</v>
+        <v>0.717674829818444</v>
       </c>
       <c r="AK74" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL74" t="b">
         <v>1</v>
@@ -8778,10 +8778,10 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="V75" t="n">
-        <v>0.5590447233485677</v>
+        <v>0.5602497627292247</v>
       </c>
       <c r="W75" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X75" t="b">
         <v>1</v>
@@ -8804,10 +8804,10 @@
         <v>0.6172839506172839</v>
       </c>
       <c r="AJ75" t="n">
-        <v>0.5794903448794144</v>
+        <v>0.5803419920136801</v>
       </c>
       <c r="AK75" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL75" t="b">
         <v>1</v>
@@ -8891,10 +8891,10 @@
         <v>0.3731343283582089</v>
       </c>
       <c r="V76" t="n">
-        <v>0.3462739704323217</v>
+        <v>0.3470203754218331</v>
       </c>
       <c r="W76" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X76" t="b">
         <v>1</v>
@@ -8917,10 +8917,10 @@
         <v>0.4065040650406504</v>
       </c>
       <c r="AJ76" t="n">
-        <v>0.3816155929693705</v>
+        <v>0.3821764337651064</v>
       </c>
       <c r="AK76" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL76" t="b">
         <v>1</v>
@@ -9004,10 +9004,10 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="V77" t="n">
-        <v>0.6489610075235122</v>
+        <v>0.6503598644269322</v>
       </c>
       <c r="W77" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X77" t="b">
         <v>1</v>
@@ -9030,10 +9030,10 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="AJ77" t="n">
-        <v>0.6519266379893413</v>
+        <v>0.6528847410153901</v>
       </c>
       <c r="AK77" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL77" t="b">
         <v>1</v>
@@ -9117,10 +9117,10 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="V78" t="n">
-        <v>0.7193908843090095</v>
+        <v>0.7209415551399323</v>
       </c>
       <c r="W78" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X78" t="b">
         <v>1</v>
@@ -9143,10 +9143,10 @@
         <v>0.7874015748031495</v>
       </c>
       <c r="AJ78" t="n">
-        <v>0.7391924084288594</v>
+        <v>0.740278761466269</v>
       </c>
       <c r="AK78" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL78" t="b">
         <v>1</v>
@@ -9230,10 +9230,10 @@
         <v>0.8</v>
       </c>
       <c r="V79" t="n">
-        <v>0.7424113926068979</v>
+        <v>0.7440116849044103</v>
       </c>
       <c r="W79" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X79" t="b">
         <v>1</v>
@@ -9256,10 +9256,10 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="AJ79" t="n">
-        <v>0.763231185938741</v>
+        <v>0.7643528675302128</v>
       </c>
       <c r="AK79" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL79" t="b">
         <v>1</v>
@@ -9343,10 +9343,10 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="V80" t="n">
-        <v>0.5693338900359647</v>
+        <v>0.5705611080555294</v>
       </c>
       <c r="W80" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X80" t="b">
         <v>1</v>
@@ -9369,10 +9369,10 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="AJ80" t="n">
-        <v>0.5830896637917089</v>
+        <v>0.5839466006597277</v>
       </c>
       <c r="AK80" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL80" t="b">
         <v>1</v>
@@ -9456,10 +9456,10 @@
         <v>0.8620689655172414</v>
       </c>
       <c r="V81" t="n">
-        <v>0.8000122765160538</v>
+        <v>0.8017367294228559</v>
       </c>
       <c r="W81" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X81" t="b">
         <v>1</v>
@@ -9482,10 +9482,10 @@
         <v>0.8695652173913044</v>
       </c>
       <c r="AJ81" t="n">
-        <v>0.8163255293083926</v>
+        <v>0.817525240923619</v>
       </c>
       <c r="AK81" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL81" t="b">
         <v>1</v>
@@ -9569,10 +9569,10 @@
         <v>0.28328611898017</v>
       </c>
       <c r="V82" t="n">
-        <v>0.2628935526228392</v>
+        <v>0.2634602283655844</v>
       </c>
       <c r="W82" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X82" t="b">
         <v>1</v>
@@ -9595,10 +9595,10 @@
         <v>0.2597402597402597</v>
       </c>
       <c r="AJ82" t="n">
-        <v>0.2438374957674419</v>
+        <v>0.2441958511849771</v>
       </c>
       <c r="AK82" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL82" t="b">
         <v>1</v>
@@ -9679,7 +9679,7 @@
       <c r="U83" t="inlineStr"/>
       <c r="V83" t="inlineStr"/>
       <c r="W83" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X83" t="b">
         <v>1</v>
@@ -9702,10 +9702,10 @@
         <v>0.2173913043478261</v>
       </c>
       <c r="AJ83" t="n">
-        <v>0.2040813823270982</v>
+        <v>0.2043813102309048</v>
       </c>
       <c r="AK83" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL83" t="b">
         <v>1</v>
@@ -9789,10 +9789,10 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="V84" t="n">
-        <v>0.4377425663955765</v>
+        <v>0.438686134967223</v>
       </c>
       <c r="W84" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X84" t="b">
         <v>1</v>
@@ -9815,10 +9815,10 @@
         <v>0.495049504950495</v>
       </c>
       <c r="AJ84" t="n">
-        <v>0.4647397815369562</v>
+        <v>0.4654227856743375</v>
       </c>
       <c r="AK84" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL84" t="b">
         <v>1</v>
@@ -9902,10 +9902,10 @@
         <v>0.2702702702702702</v>
       </c>
       <c r="V85" t="n">
-        <v>0.2508146596644925</v>
+        <v>0.2513552989541926</v>
       </c>
       <c r="W85" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X85" t="b">
         <v>1</v>
@@ -9928,10 +9928,10 @@
         <v>0.2380952380952381</v>
       </c>
       <c r="AJ85" t="n">
-        <v>0.2235177044534884</v>
+        <v>0.2238461969195623</v>
       </c>
       <c r="AK85" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL85" t="b">
         <v>1</v>
@@ -10015,10 +10015,10 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="V86" t="n">
-        <v>0.3834769589911663</v>
+        <v>0.384303556252278</v>
       </c>
       <c r="W86" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X86" t="b">
         <v>1</v>
@@ -10041,10 +10041,10 @@
         <v>0.390625</v>
       </c>
       <c r="AJ86" t="n">
-        <v>0.3667087338690045</v>
+        <v>0.3672476668211569</v>
       </c>
       <c r="AK86" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL86" t="b">
         <v>1</v>
@@ -10125,7 +10125,7 @@
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X87" t="b">
         <v>1</v>
@@ -10148,10 +10148,10 @@
         <v>0.4201680672268908</v>
       </c>
       <c r="AJ87" t="n">
-        <v>0.3944430078590972</v>
+        <v>0.3950227004462865</v>
       </c>
       <c r="AK87" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL87" t="b">
         <v>1</v>
@@ -10235,10 +10235,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="V88" t="n">
-        <v>0.5213563150329339</v>
+        <v>0.5224801158036589</v>
       </c>
       <c r="W88" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X88" t="b">
         <v>1</v>
@@ -10261,10 +10261,10 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="AJ88" t="n">
-        <v>0.5274013251149727</v>
+        <v>0.5281764196978437</v>
       </c>
       <c r="AK88" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL88" t="b">
         <v>1</v>
@@ -10362,10 +10362,10 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="AJ89" t="n">
-        <v>0.7277320610113577</v>
+        <v>0.7288015713660168</v>
       </c>
       <c r="AK89" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL89" t="b">
         <v>1</v>
@@ -10463,10 +10463,10 @@
         <v>0.3968253968253968</v>
       </c>
       <c r="AJ90" t="n">
-        <v>0.3725295074224807</v>
+        <v>0.3730769948659372</v>
       </c>
       <c r="AK90" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL90" t="b">
         <v>1</v>
@@ -10547,7 +10547,7 @@
       <c r="U91" t="inlineStr"/>
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X91" t="b">
         <v>1</v>
@@ -10570,10 +10570,10 @@
         <v>0.5586592178770949</v>
       </c>
       <c r="AJ91" t="n">
-        <v>0.5244549489970119</v>
+        <v>0.5252257134425484</v>
       </c>
       <c r="AK91" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL91" t="b">
         <v>1</v>
@@ -10657,10 +10657,10 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="V92" t="n">
-        <v>0.7544831225679857</v>
+        <v>0.7561094358784657</v>
       </c>
       <c r="W92" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X92" t="b">
         <v>1</v>
@@ -10683,10 +10683,10 @@
         <v>0.8264462809917356</v>
       </c>
       <c r="AJ92" t="n">
-        <v>0.7758465774418607</v>
+        <v>0.7769867992249271</v>
       </c>
       <c r="AK92" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="AL92" t="b">
         <v>1</v>
@@ -10770,10 +10770,10 @@
         <v>0.2932551319648093</v>
       </c>
       <c r="V93" t="n">
-        <v>0.2721449386388922</v>
+        <v>0.2727315560500037</v>
       </c>
       <c r="W93" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X93" t="b">
         <v>1</v>
@@ -10871,10 +10871,10 @@
         <v>0.53475935828877</v>
       </c>
       <c r="V94" t="n">
-        <v>0.496264299870921</v>
+        <v>0.4973340139735362</v>
       </c>
       <c r="W94" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="X94" t="b">
         <v>1</v>
@@ -11332,7 +11332,7 @@
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z4" t="b">
         <v>1</v>
@@ -11417,13 +11417,13 @@
         <v>0.819672131147541</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z5" t="b">
         <v>1</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.7694871792661078</v>
+        <v>0.7706180549689851</v>
       </c>
     </row>
     <row r="6">
@@ -11504,13 +11504,13 @@
         <v>0.8</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z6" t="b">
         <v>1</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.7424113926068979</v>
+        <v>0.7440116849044103</v>
       </c>
     </row>
     <row r="7">
@@ -11591,13 +11591,13 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z7" t="b">
         <v>1</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.496706009896641</v>
+        <v>0.497435993154583</v>
       </c>
     </row>
     <row r="8">
@@ -11678,13 +11678,13 @@
         <v>0.4901960784313725</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z8" t="b">
         <v>1</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.4549089415483443</v>
+        <v>0.4558895128090749</v>
       </c>
     </row>
     <row r="9">
@@ -11765,13 +11765,13 @@
         <v>0.4464285714285714</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z9" t="b">
         <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.4190956958502908</v>
+        <v>0.4197116192241793</v>
       </c>
     </row>
     <row r="10">
@@ -11844,7 +11844,7 @@
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z10" t="b">
         <v>1</v>
@@ -11929,13 +11929,13 @@
         <v>0.4975124378109453</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z11" t="b">
         <v>1</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.4616986272430957</v>
+        <v>0.4626938338957776</v>
       </c>
     </row>
     <row r="12">
@@ -12016,13 +12016,13 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z12" t="b">
         <v>1</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.6852367581785777</v>
+        <v>0.6862438153738407</v>
       </c>
     </row>
     <row r="13">
@@ -12103,13 +12103,13 @@
         <v>0.5464480874316939</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z13" t="b">
         <v>1</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.5129914528440718</v>
+        <v>0.5137453699793233</v>
       </c>
     </row>
     <row r="14">
@@ -12190,13 +12190,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z14" t="b">
         <v>1</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.5624328731870438</v>
+        <v>0.5636452158366745</v>
       </c>
     </row>
     <row r="15">
@@ -12277,13 +12277,13 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z15" t="b">
         <v>1</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.7733452006321854</v>
+        <v>0.7750121717754274</v>
       </c>
     </row>
     <row r="16">
@@ -12364,13 +12364,13 @@
         <v>0.5952380952380952</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z16" t="b">
         <v>1</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.5587942611337211</v>
+        <v>0.5596154922989058</v>
       </c>
     </row>
     <row r="17">
@@ -12451,13 +12451,13 @@
         <v>0.6451612903225806</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z17" t="b">
         <v>1</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.5987188650055628</v>
+        <v>0.6000094233100083</v>
       </c>
     </row>
     <row r="18">
@@ -12538,13 +12538,13 @@
         <v>0.5681818181818182</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z18" t="b">
         <v>1</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.5333945219912792</v>
+        <v>0.5341784244671374</v>
       </c>
     </row>
     <row r="19">
@@ -12625,13 +12625,13 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z19" t="b">
         <v>1</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.4571498722948879</v>
+        <v>0.4581352739559177</v>
       </c>
     </row>
     <row r="20">
@@ -12712,13 +12712,13 @@
         <v>0.3802281368821293</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z20" t="b">
         <v>1</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.3528571257637347</v>
+        <v>0.3536177209621722</v>
       </c>
     </row>
     <row r="21">
@@ -12799,13 +12799,13 @@
         <v>0.4065040650406504</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z21" t="b">
         <v>1</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.3816155929693705</v>
+        <v>0.3821764337651064</v>
       </c>
     </row>
     <row r="22">
@@ -12886,13 +12886,13 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z22" t="b">
         <v>1</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.7277320610113577</v>
+        <v>0.7288015713660168</v>
       </c>
     </row>
     <row r="23">
@@ -12973,13 +12973,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z23" t="b">
         <v>1</v>
       </c>
       <c r="AA23" t="n">
-        <v>0.5689541567906978</v>
+        <v>0.5697903194316132</v>
       </c>
     </row>
     <row r="24">
@@ -13060,13 +13060,13 @@
         <v>0.6289308176100629</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z24" t="b">
         <v>1</v>
       </c>
       <c r="AA24" t="n">
-        <v>0.5836567551941021</v>
+        <v>0.584914846622964</v>
       </c>
     </row>
     <row r="25">
@@ -13147,13 +13147,13 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z25" t="b">
         <v>1</v>
       </c>
       <c r="AA25" t="n">
-        <v>0.4470354089069768</v>
+        <v>0.4476923938391246</v>
       </c>
     </row>
     <row r="26">
@@ -13234,13 +13234,13 @@
         <v>0.6578947368421053</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z26" t="b">
         <v>1</v>
       </c>
       <c r="AA26" t="n">
-        <v>0.6176147096741128</v>
+        <v>0.6185223862251065</v>
       </c>
     </row>
     <row r="27">
@@ -13321,13 +13321,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z27" t="b">
         <v>1</v>
       </c>
       <c r="AA27" t="n">
-        <v>0.6186761605057483</v>
+        <v>0.6200097374203418</v>
       </c>
     </row>
     <row r="28">
@@ -13408,13 +13408,13 @@
         <v>0.3571428571428572</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z28" t="b">
         <v>1</v>
       </c>
       <c r="AA28" t="n">
-        <v>0.3352765566802327</v>
+        <v>0.3357692953793435</v>
       </c>
     </row>
     <row r="29">
@@ -13487,7 +13487,7 @@
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
       <c r="Y29" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z29" t="b">
         <v>1</v>
@@ -13572,13 +13572,13 @@
         <v>0.9174311926605504</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z30" t="b">
         <v>1</v>
       </c>
       <c r="AA30" t="n">
-        <v>0.8612608795455517</v>
+        <v>0.8625266303322584</v>
       </c>
     </row>
     <row r="31">
@@ -13659,13 +13659,13 @@
         <v>0.8928571428571428</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z31" t="b">
         <v>1</v>
       </c>
       <c r="AA31" t="n">
-        <v>0.8285841435344842</v>
+        <v>0.8303701840451007</v>
       </c>
     </row>
     <row r="32">
@@ -13746,13 +13746,13 @@
         <v>0.4273504273504274</v>
       </c>
       <c r="Y32" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z32" t="b">
         <v>1</v>
       </c>
       <c r="AA32" t="n">
-        <v>0.4011856233780562</v>
+        <v>0.4017752252402401</v>
       </c>
     </row>
     <row r="33">
@@ -13833,13 +13833,13 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z33" t="b">
         <v>1</v>
       </c>
       <c r="AA33" t="n">
-        <v>0.4316345305854057</v>
+        <v>0.4325649330839594</v>
       </c>
     </row>
     <row r="34">
@@ -13920,13 +13920,13 @@
         <v>0.4587155963302752</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z34" t="b">
         <v>1</v>
       </c>
       <c r="AA34" t="n">
-        <v>0.4306304397727759</v>
+        <v>0.4312633151661292</v>
       </c>
     </row>
     <row r="35">
@@ -14007,13 +14007,13 @@
         <v>0.4566210045662101</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z35" t="b">
         <v>1</v>
       </c>
       <c r="AA35" t="n">
-        <v>0.4237507948669509</v>
+        <v>0.424664203712563</v>
       </c>
     </row>
     <row r="36">
@@ -14094,13 +14094,13 @@
         <v>0.495049504950495</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z36" t="b">
         <v>1</v>
       </c>
       <c r="AA36" t="n">
-        <v>0.4647397815369562</v>
+        <v>0.4654227856743375</v>
       </c>
     </row>
     <row r="37">
@@ -14181,13 +14181,13 @@
         <v>0.4694835680751174</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z37" t="b">
         <v>1</v>
       </c>
       <c r="AA37" t="n">
-        <v>0.435687436975879</v>
+        <v>0.4366265756481281</v>
       </c>
     </row>
     <row r="38">
@@ -14268,13 +14268,13 @@
         <v>0.625</v>
       </c>
       <c r="Y38" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z38" t="b">
         <v>1</v>
       </c>
       <c r="AA38" t="n">
-        <v>0.5867339741904072</v>
+        <v>0.5875962669138511</v>
       </c>
     </row>
     <row r="39">
@@ -14355,13 +14355,13 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z39" t="b">
         <v>1</v>
       </c>
       <c r="AA39" t="n">
-        <v>0.5693338900359647</v>
+        <v>0.5705611080555294</v>
       </c>
     </row>
     <row r="40">
@@ -14442,13 +14442,13 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="Y40" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z40" t="b">
         <v>1</v>
       </c>
       <c r="AA40" t="n">
-        <v>0.5655267221112359</v>
+        <v>0.5663578476278083</v>
       </c>
     </row>
     <row r="41">
@@ -14529,13 +14529,13 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z41" t="b">
         <v>1</v>
       </c>
       <c r="AA41" t="n">
-        <v>0.5302938518620699</v>
+        <v>0.5314369177888645</v>
       </c>
     </row>
     <row r="42">
@@ -14616,13 +14616,13 @@
         <v>0.8474576271186441</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z42" t="b">
         <v>1</v>
       </c>
       <c r="AA42" t="n">
-        <v>0.7955714904276707</v>
+        <v>0.7967407009001372</v>
       </c>
     </row>
     <row r="43">
@@ -14703,13 +14703,13 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z43" t="b">
         <v>1</v>
       </c>
       <c r="AA43" t="n">
-        <v>0.7733452006321854</v>
+        <v>0.7750121717754274</v>
       </c>
     </row>
     <row r="44">
@@ -14790,13 +14790,13 @@
         <v>0.4545454545454545</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z44" t="b">
         <v>1</v>
       </c>
       <c r="AA44" t="n">
-        <v>0.4267156175930233</v>
+        <v>0.4273427395737099</v>
       </c>
     </row>
     <row r="45">
@@ -14877,13 +14877,13 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z45" t="b">
         <v>1</v>
       </c>
       <c r="AA45" t="n">
-        <v>0.4377425663955765</v>
+        <v>0.438686134967223</v>
       </c>
     </row>
     <row r="46">
@@ -14964,13 +14964,13 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z46" t="b">
         <v>1</v>
       </c>
       <c r="AA46" t="n">
-        <v>0.6657974175210294</v>
+        <v>0.6667759057178453</v>
       </c>
     </row>
     <row r="47">
@@ -15051,13 +15051,13 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z47" t="b">
         <v>1</v>
       </c>
       <c r="AA47" t="n">
-        <v>0.6444543338601544</v>
+        <v>0.6458434764795228</v>
       </c>
     </row>
     <row r="48">
@@ -15138,13 +15138,13 @@
         <v>0.3968253968253968</v>
       </c>
       <c r="Y48" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z48" t="b">
         <v>1</v>
       </c>
       <c r="AA48" t="n">
-        <v>0.3725295074224807</v>
+        <v>0.3730769948659372</v>
       </c>
     </row>
     <row r="49">
@@ -15225,13 +15225,13 @@
         <v>0.3759398496240601</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z49" t="b">
         <v>1</v>
       </c>
       <c r="AA49" t="n">
-        <v>0.3488775341197828</v>
+        <v>0.3496295511768845</v>
       </c>
     </row>
     <row r="50">
@@ -15312,13 +15312,13 @@
         <v>0.4672897196261682</v>
       </c>
       <c r="Y50" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z50" t="b">
         <v>1</v>
       </c>
       <c r="AA50" t="n">
-        <v>0.4386796068713325</v>
+        <v>0.4393243117112905</v>
       </c>
     </row>
     <row r="51">
@@ -15399,13 +15399,13 @@
         <v>0.4629629629629629</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z51" t="b">
         <v>1</v>
       </c>
       <c r="AA51" t="n">
-        <v>0.4296362225734362</v>
+        <v>0.4305623176530151</v>
       </c>
     </row>
     <row r="52">
@@ -15486,13 +15486,13 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="Y52" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z52" t="b">
         <v>1</v>
       </c>
       <c r="AA52" t="n">
-        <v>0.6217048733143388</v>
+        <v>0.6226185609683191</v>
       </c>
     </row>
     <row r="53">
@@ -15573,13 +15573,13 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z53" t="b">
         <v>1</v>
       </c>
       <c r="AA53" t="n">
-        <v>0.6270366491612313</v>
+        <v>0.6283882473854816</v>
       </c>
     </row>
     <row r="54">
@@ -15660,13 +15660,13 @@
         <v>0.5319148936170213</v>
       </c>
       <c r="Y54" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z54" t="b">
         <v>1</v>
       </c>
       <c r="AA54" t="n">
-        <v>0.499348063140772</v>
+        <v>0.5000819292883839</v>
       </c>
     </row>
     <row r="55">
@@ -15747,13 +15747,13 @@
         <v>0.5291005291005292</v>
       </c>
       <c r="Y55" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z55" t="b">
         <v>1</v>
       </c>
       <c r="AA55" t="n">
-        <v>0.491012825798213</v>
+        <v>0.4920712201748746</v>
       </c>
     </row>
     <row r="56">
@@ -15834,13 +15834,13 @@
         <v>0.8264462809917356</v>
       </c>
       <c r="Y56" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z56" t="b">
         <v>1</v>
       </c>
       <c r="AA56" t="n">
-        <v>0.7758465774418607</v>
+        <v>0.7769867992249271</v>
       </c>
     </row>
     <row r="57">
@@ -15913,7 +15913,7 @@
       <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr"/>
       <c r="Y57" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z57" t="b">
         <v>1</v>
@@ -15998,13 +15998,13 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="Y58" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z58" t="b">
         <v>1</v>
       </c>
       <c r="AA58" t="n">
-        <v>0.763231185938741</v>
+        <v>0.7643528675302128</v>
       </c>
     </row>
     <row r="59">
@@ -16085,13 +16085,13 @@
         <v>0.8</v>
       </c>
       <c r="Y59" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z59" t="b">
         <v>1</v>
       </c>
       <c r="AA59" t="n">
-        <v>0.7424113926068979</v>
+        <v>0.7440116849044103</v>
       </c>
     </row>
     <row r="60">
@@ -16172,13 +16172,13 @@
         <v>0.6756756756756757</v>
       </c>
       <c r="Y60" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z60" t="b">
         <v>1</v>
       </c>
       <c r="AA60" t="n">
-        <v>0.6343069991247645</v>
+        <v>0.6352392074744336</v>
       </c>
     </row>
     <row r="61">
@@ -16259,13 +16259,13 @@
         <v>0.4347826086956522</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z61" t="b">
         <v>1</v>
       </c>
       <c r="AA61" t="n">
-        <v>0.4081627646541963</v>
+        <v>0.4087626204618095</v>
       </c>
     </row>
     <row r="62">
@@ -16346,13 +16346,13 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="Y62" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z62" t="b">
         <v>1</v>
       </c>
       <c r="AA62" t="n">
-        <v>0.3932263732028061</v>
+        <v>0.3940739856485224</v>
       </c>
     </row>
     <row r="63">
@@ -16433,13 +16433,13 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="Y63" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z63" t="b">
         <v>1</v>
       </c>
       <c r="AA63" t="n">
-        <v>0.5873507852902673</v>
+        <v>0.5886168393231093</v>
       </c>
     </row>
     <row r="64">
@@ -16520,13 +16520,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y64" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z64" t="b">
         <v>1</v>
       </c>
       <c r="AA64" t="n">
-        <v>0.7058453824847003</v>
+        <v>0.7068827271144072</v>
       </c>
     </row>
     <row r="65">
@@ -16607,13 +16607,13 @@
         <v>0.9345794392523364</v>
       </c>
       <c r="Y65" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z65" t="b">
         <v>1</v>
       </c>
       <c r="AA65" t="n">
-        <v>0.8773592137426649</v>
+        <v>0.8786486234225811</v>
       </c>
     </row>
     <row r="66">
@@ -16694,13 +16694,13 @@
         <v>0.6097560975609756</v>
       </c>
       <c r="Y66" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z66" t="b">
         <v>1</v>
       </c>
       <c r="AA66" t="n">
-        <v>0.5724233894540557</v>
+        <v>0.5732646506476596</v>
       </c>
     </row>
     <row r="67">
@@ -16781,13 +16781,13 @@
         <v>0.591715976331361</v>
       </c>
       <c r="Y67" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z67" t="b">
         <v>1</v>
       </c>
       <c r="AA67" t="n">
-        <v>0.549120852519895</v>
+        <v>0.5503045006689425</v>
       </c>
     </row>
     <row r="68">
@@ -16868,13 +16868,13 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z68" t="b">
         <v>1</v>
       </c>
       <c r="AA68" t="n">
-        <v>0.763231185938741</v>
+        <v>0.7643528675302128</v>
       </c>
     </row>
     <row r="69">
@@ -16955,13 +16955,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y69" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z69" t="b">
         <v>1</v>
       </c>
       <c r="AA69" t="n">
-        <v>0.7058453824847003</v>
+        <v>0.7068827271144072</v>
       </c>
     </row>
     <row r="70">
@@ -17042,13 +17042,13 @@
         <v>0.8064516129032259</v>
       </c>
       <c r="Y70" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z70" t="b">
         <v>1</v>
       </c>
       <c r="AA70" t="n">
-        <v>0.7483985812569536</v>
+        <v>0.7500117791375104</v>
       </c>
     </row>
     <row r="71">
@@ -17129,13 +17129,13 @@
         <v>0.8</v>
       </c>
       <c r="Y71" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z71" t="b">
         <v>1</v>
       </c>
       <c r="AA71" t="n">
-        <v>0.7510194869637212</v>
+        <v>0.7521232216497294</v>
       </c>
     </row>
     <row r="72">
@@ -17208,7 +17208,7 @@
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr"/>
       <c r="Y72" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z72" t="b">
         <v>1</v>
@@ -17293,13 +17293,13 @@
         <v>0.8264462809917356</v>
       </c>
       <c r="Y73" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z73" t="b">
         <v>1</v>
       </c>
       <c r="AA73" t="n">
-        <v>0.7758465774418607</v>
+        <v>0.7769867992249271</v>
       </c>
     </row>
     <row r="74">
@@ -17372,7 +17372,7 @@
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr"/>
       <c r="Y74" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z74" t="b">
         <v>1</v>
@@ -17457,13 +17457,13 @@
         <v>0.8403361344537815</v>
       </c>
       <c r="Y75" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z75" t="b">
         <v>1</v>
       </c>
       <c r="AA75" t="n">
-        <v>0.7888860157181945</v>
+        <v>0.7900454008925729</v>
       </c>
     </row>
     <row r="76">
@@ -17536,7 +17536,7 @@
       <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr"/>
       <c r="Y76" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z76" t="b">
         <v>1</v>
@@ -17621,13 +17621,13 @@
         <v>0.591715976331361</v>
       </c>
       <c r="Y77" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z77" t="b">
         <v>1</v>
       </c>
       <c r="AA77" t="n">
-        <v>0.5554877862157701</v>
+        <v>0.5563041580249478</v>
       </c>
     </row>
     <row r="78">
@@ -17708,13 +17708,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="Y78" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z78" t="b">
         <v>1</v>
       </c>
       <c r="AA78" t="n">
-        <v>0.6186761605057483</v>
+        <v>0.6200097374203418</v>
       </c>
     </row>
     <row r="79">
@@ -17795,13 +17795,13 @@
         <v>0.4464285714285714</v>
       </c>
       <c r="Y79" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z79" t="b">
         <v>1</v>
       </c>
       <c r="AA79" t="n">
-        <v>0.4190956958502908</v>
+        <v>0.4197116192241793</v>
       </c>
     </row>
     <row r="80">
@@ -17882,13 +17882,13 @@
         <v>0.4761904761904762</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z80" t="b">
         <v>1</v>
       </c>
       <c r="AA80" t="n">
-        <v>0.4419115432183915</v>
+        <v>0.442864098157387</v>
       </c>
     </row>
     <row r="81">
@@ -17969,13 +17969,13 @@
         <v>0.4065040650406504</v>
       </c>
       <c r="Y81" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z81" t="b">
         <v>1</v>
       </c>
       <c r="AA81" t="n">
-        <v>0.3816155929693705</v>
+        <v>0.3821764337651064</v>
       </c>
     </row>
     <row r="82">
@@ -18056,13 +18056,13 @@
         <v>0.4237288135593221</v>
       </c>
       <c r="Y82" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z82" t="b">
         <v>1</v>
       </c>
       <c r="AA82" t="n">
-        <v>0.3932263732028061</v>
+        <v>0.3940739856485224</v>
       </c>
     </row>
     <row r="83">
@@ -18143,13 +18143,13 @@
         <v>0.5102040816326531</v>
       </c>
       <c r="Y83" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z83" t="b">
         <v>1</v>
       </c>
       <c r="AA83" t="n">
-        <v>0.4789665095431895</v>
+        <v>0.4796704219704907</v>
       </c>
     </row>
     <row r="84">
@@ -18230,13 +18230,13 @@
         <v>0.5</v>
       </c>
       <c r="Y84" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z84" t="b">
         <v>1</v>
       </c>
       <c r="AA84" t="n">
-        <v>0.4640071203793112</v>
+        <v>0.4650073030652564</v>
       </c>
     </row>
     <row r="85">
@@ -18317,13 +18317,13 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="Y85" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z85" t="b">
         <v>1</v>
       </c>
       <c r="AA85" t="n">
-        <v>0.5522202110027361</v>
+        <v>0.5530317806248011</v>
       </c>
     </row>
     <row r="86">
@@ -18396,7 +18396,7 @@
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr"/>
       <c r="Y86" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z86" t="b">
         <v>1</v>
@@ -18481,13 +18481,13 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="Y87" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z87" t="b">
         <v>1</v>
       </c>
       <c r="AA87" t="n">
-        <v>0.7277320610113577</v>
+        <v>0.7288015713660168</v>
       </c>
     </row>
     <row r="88">
@@ -18568,13 +18568,13 @@
         <v>0.5494505494505494</v>
       </c>
       <c r="Y88" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z88" t="b">
         <v>1</v>
       </c>
       <c r="AA88" t="n">
-        <v>0.5158100872003578</v>
+        <v>0.5165681467374514</v>
       </c>
     </row>
     <row r="89">
@@ -18655,13 +18655,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z89" t="b">
         <v>1</v>
       </c>
       <c r="AA89" t="n">
-        <v>0.5213563150329339</v>
+        <v>0.5224801158036589</v>
       </c>
     </row>
     <row r="90">
@@ -18742,13 +18742,13 @@
         <v>0.5988023952095809</v>
       </c>
       <c r="Y90" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z90" t="b">
         <v>1</v>
       </c>
       <c r="AA90" t="n">
-        <v>0.5621403345536835</v>
+        <v>0.5629664832707556</v>
       </c>
     </row>
     <row r="91">
@@ -18829,13 +18829,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z91" t="b">
         <v>1</v>
       </c>
       <c r="AA91" t="n">
-        <v>0.5624328731870438</v>
+        <v>0.5636452158366745</v>
       </c>
     </row>
     <row r="92">
@@ -18916,13 +18916,13 @@
         <v>0.5988023952095809</v>
       </c>
       <c r="Y92" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z92" t="b">
         <v>1</v>
       </c>
       <c r="AA92" t="n">
-        <v>0.5621403345536835</v>
+        <v>0.5629664832707556</v>
       </c>
     </row>
     <row r="93">
@@ -19003,13 +19003,13 @@
         <v>0.5882352941176471</v>
       </c>
       <c r="Y93" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z93" t="b">
         <v>1</v>
       </c>
       <c r="AA93" t="n">
-        <v>0.5458907298580131</v>
+        <v>0.5470674153708899</v>
       </c>
     </row>
     <row r="94">
@@ -19090,13 +19090,13 @@
         <v>0.6578947368421053</v>
       </c>
       <c r="Y94" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z94" t="b">
         <v>1</v>
       </c>
       <c r="AA94" t="n">
-        <v>0.6176147096741128</v>
+        <v>0.6185223862251065</v>
       </c>
     </row>
     <row r="95">
@@ -19177,13 +19177,13 @@
         <v>0.6622516556291391</v>
       </c>
       <c r="Y95" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z95" t="b">
         <v>1</v>
       </c>
       <c r="AA95" t="n">
-        <v>0.6145789673898162</v>
+        <v>0.6159037126692138</v>
       </c>
     </row>
     <row r="96">
@@ -19264,13 +19264,13 @@
         <v>0.6329113924050632</v>
       </c>
       <c r="Y96" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z96" t="b">
         <v>1</v>
       </c>
       <c r="AA96" t="n">
-        <v>0.5941609865219312</v>
+        <v>0.5950341943431403</v>
       </c>
     </row>
     <row r="97">
@@ -19351,13 +19351,13 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="Y97" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z97" t="b">
         <v>1</v>
       </c>
       <c r="AA97" t="n">
-        <v>0.5910918730946639</v>
+        <v>0.5923659911659317</v>
       </c>
     </row>
     <row r="98">
@@ -19438,13 +19438,13 @@
         <v>0.4672897196261682</v>
       </c>
       <c r="Y98" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z98" t="b">
         <v>1</v>
       </c>
       <c r="AA98" t="n">
-        <v>0.4386796068713325</v>
+        <v>0.4393243117112905</v>
       </c>
     </row>
     <row r="99">
@@ -19525,13 +19525,13 @@
         <v>0.4651162790697674</v>
       </c>
       <c r="Y99" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z99" t="b">
         <v>1</v>
       </c>
       <c r="AA99" t="n">
-        <v>0.4316345305854057</v>
+        <v>0.4325649330839594</v>
       </c>
     </row>
     <row r="100">
@@ -19612,13 +19612,13 @@
         <v>0.7692307692307692</v>
       </c>
       <c r="Y100" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z100" t="b">
         <v>1</v>
       </c>
       <c r="AA100" t="n">
-        <v>0.722134122080501</v>
+        <v>0.723195405432432</v>
       </c>
     </row>
     <row r="101">
@@ -19699,13 +19699,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y101" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z101" t="b">
         <v>1</v>
       </c>
       <c r="AA101" t="n">
-        <v>0.6977550682395657</v>
+        <v>0.699259102353769</v>
       </c>
     </row>
     <row r="102">
@@ -19786,13 +19786,13 @@
         <v>0.495049504950495</v>
       </c>
       <c r="Y102" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z102" t="b">
         <v>1</v>
       </c>
       <c r="AA102" t="n">
-        <v>0.4647397815369562</v>
+        <v>0.4654227856743375</v>
       </c>
     </row>
     <row r="103">
@@ -19873,13 +19873,13 @@
         <v>0.4926108374384237</v>
       </c>
       <c r="Y103" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z103" t="b">
         <v>1</v>
       </c>
       <c r="AA103" t="n">
-        <v>0.4571498722948879</v>
+        <v>0.4581352739559177</v>
       </c>
     </row>
     <row r="104">
@@ -19960,13 +19960,13 @@
         <v>0.6097560975609756</v>
       </c>
       <c r="Y104" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z104" t="b">
         <v>1</v>
       </c>
       <c r="AA104" t="n">
-        <v>0.5724233894540557</v>
+        <v>0.5732646506476596</v>
       </c>
     </row>
     <row r="105">
@@ -20047,13 +20047,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y105" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z105" t="b">
         <v>1</v>
       </c>
       <c r="AA105" t="n">
-        <v>0.5764063607196411</v>
+        <v>0.5776488236835483</v>
       </c>
     </row>
     <row r="106">
@@ -20134,13 +20134,13 @@
         <v>0.7692307692307692</v>
       </c>
       <c r="Y106" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z106" t="b">
         <v>1</v>
       </c>
       <c r="AA106" t="n">
-        <v>0.722134122080501</v>
+        <v>0.723195405432432</v>
       </c>
     </row>
     <row r="107">
@@ -20221,13 +20221,13 @@
         <v>0.7518796992481203</v>
       </c>
       <c r="Y107" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z107" t="b">
         <v>1</v>
       </c>
       <c r="AA107" t="n">
-        <v>0.6977550682395657</v>
+        <v>0.699259102353769</v>
       </c>
     </row>
     <row r="108">
@@ -20308,13 +20308,13 @@
         <v>0.3472222222222222</v>
       </c>
       <c r="Y108" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z108" t="b">
         <v>1</v>
       </c>
       <c r="AA108" t="n">
-        <v>0.3259633189946706</v>
+        <v>0.326442370507695</v>
       </c>
     </row>
     <row r="109">
@@ -20387,7 +20387,7 @@
       <c r="W109" t="inlineStr"/>
       <c r="X109" t="inlineStr"/>
       <c r="Y109" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z109" t="b">
         <v>1</v>
@@ -20472,13 +20472,13 @@
         <v>0.6060606060606061</v>
       </c>
       <c r="Y110" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z110" t="b">
         <v>1</v>
       </c>
       <c r="AA110" t="n">
-        <v>0.5689541567906978</v>
+        <v>0.5697903194316132</v>
       </c>
     </row>
     <row r="111">
@@ -20559,13 +20559,13 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="Y111" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z111" t="b">
         <v>1</v>
       </c>
       <c r="AA111" t="n">
-        <v>0.3879232887209303</v>
+        <v>0.3884933996124635</v>
       </c>
     </row>
     <row r="112">
@@ -20646,13 +20646,13 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="Y112" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z112" t="b">
         <v>1</v>
       </c>
       <c r="AA112" t="n">
-        <v>0.3866726003160927</v>
+        <v>0.3875060858877137</v>
       </c>
     </row>
     <row r="113">
@@ -20733,13 +20733,13 @@
         <v>0.7407407407407407</v>
       </c>
       <c r="Y113" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z113" t="b">
         <v>1</v>
       </c>
       <c r="AA113" t="n">
-        <v>0.6953884138552974</v>
+        <v>0.6964103904164161</v>
       </c>
     </row>
     <row r="114">
@@ -20820,13 +20820,13 @@
         <v>0.7299270072992701</v>
       </c>
       <c r="Y114" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z114" t="b">
         <v>1</v>
       </c>
       <c r="AA114" t="n">
-        <v>0.6773826574880455</v>
+        <v>0.6788427781974546</v>
       </c>
     </row>
     <row r="115">
@@ -20907,13 +20907,13 @@
         <v>0.8849557522123894</v>
       </c>
       <c r="Y115" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z115" t="b">
         <v>1</v>
       </c>
       <c r="AA115" t="n">
-        <v>0.8307737687651783</v>
+        <v>0.8319947142143025</v>
       </c>
     </row>
     <row r="116">
@@ -20986,7 +20986,7 @@
       <c r="W116" t="inlineStr"/>
       <c r="X116" t="inlineStr"/>
       <c r="Y116" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z116" t="b">
         <v>1</v>
@@ -21071,13 +21071,13 @@
         <v>0.3378378378378378</v>
       </c>
       <c r="Y117" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z117" t="b">
         <v>1</v>
       </c>
       <c r="AA117" t="n">
-        <v>0.3171534995623823</v>
+        <v>0.3176196037372168</v>
       </c>
     </row>
     <row r="118">
@@ -21158,13 +21158,13 @@
         <v>0.3521126760563381</v>
       </c>
       <c r="Y118" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z118" t="b">
         <v>1</v>
       </c>
       <c r="AA118" t="n">
-        <v>0.3267655777319093</v>
+        <v>0.3274699317360961</v>
       </c>
     </row>
     <row r="119">
@@ -21245,13 +21245,13 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="Y119" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z119" t="b">
         <v>1</v>
       </c>
       <c r="AA119" t="n">
-        <v>0.6657974175210294</v>
+        <v>0.6667759057178453</v>
       </c>
     </row>
     <row r="120">
@@ -21332,13 +21332,13 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="Y120" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z120" t="b">
         <v>1</v>
       </c>
       <c r="AA120" t="n">
-        <v>0.6489610075235122</v>
+        <v>0.6503598644269322</v>
       </c>
     </row>
     <row r="121">
@@ -21419,13 +21419,13 @@
         <v>0.6369426751592356</v>
       </c>
       <c r="Y121" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z121" t="b">
         <v>1</v>
       </c>
       <c r="AA121" t="n">
-        <v>0.5979454514042366</v>
+        <v>0.5988242210587017</v>
       </c>
     </row>
     <row r="122">
@@ -21506,13 +21506,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y122" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z122" t="b">
         <v>1</v>
       </c>
       <c r="AA122" t="n">
-        <v>0.5764063607196411</v>
+        <v>0.5776488236835483</v>
       </c>
     </row>
     <row r="123">
@@ -21593,13 +21593,13 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="Y123" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z123" t="b">
         <v>1</v>
       </c>
       <c r="AA123" t="n">
-        <v>0.6519266379893413</v>
+        <v>0.6528847410153901</v>
       </c>
     </row>
     <row r="124">
@@ -21672,7 +21672,7 @@
       <c r="W124" t="inlineStr"/>
       <c r="X124" t="inlineStr"/>
       <c r="Y124" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z124" t="b">
         <v>1</v>
@@ -21757,13 +21757,13 @@
         <v>0.8771929824561404</v>
       </c>
       <c r="Y125" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z125" t="b">
         <v>1</v>
       </c>
       <c r="AA125" t="n">
-        <v>0.8234862795654838</v>
+        <v>0.8246965149668086</v>
       </c>
     </row>
     <row r="126">
@@ -21844,13 +21844,13 @@
         <v>0.8547008547008548</v>
       </c>
       <c r="Y126" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z126" t="b">
         <v>1</v>
       </c>
       <c r="AA126" t="n">
-        <v>0.7931745647509594</v>
+        <v>0.7948842787440281</v>
       </c>
     </row>
     <row r="127">
@@ -21931,13 +21931,13 @@
         <v>0.7042253521126761</v>
       </c>
       <c r="Y127" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z127" t="b">
         <v>1</v>
       </c>
       <c r="AA127" t="n">
-        <v>0.6611087033131349</v>
+        <v>0.6620803007480013</v>
       </c>
     </row>
     <row r="128">
@@ -22018,13 +22018,13 @@
         <v>0.7092198581560284</v>
       </c>
       <c r="Y128" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z128" t="b">
         <v>1</v>
       </c>
       <c r="AA128" t="n">
-        <v>0.6581661281976046</v>
+        <v>0.6595848270429169</v>
       </c>
     </row>
     <row r="129">
@@ -22105,13 +22105,13 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="Y129" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z129" t="b">
         <v>1</v>
       </c>
       <c r="AA129" t="n">
-        <v>0.7166216478661461</v>
+        <v>0.717674829818444</v>
       </c>
     </row>
     <row r="130">
@@ -22192,13 +22192,13 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="Y130" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z130" t="b">
         <v>1</v>
       </c>
       <c r="AA130" t="n">
-        <v>0.7084078173729941</v>
+        <v>0.7099348138400861</v>
       </c>
     </row>
     <row r="131">
@@ -22279,13 +22279,13 @@
         <v>0.6172839506172839</v>
       </c>
       <c r="Y131" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z131" t="b">
         <v>1</v>
       </c>
       <c r="AA131" t="n">
-        <v>0.5794903448794144</v>
+        <v>0.5803419920136801</v>
       </c>
     </row>
     <row r="132">
@@ -22366,13 +22366,13 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="Y132" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z132" t="b">
         <v>1</v>
       </c>
       <c r="AA132" t="n">
-        <v>0.5590447233485677</v>
+        <v>0.5602497627292247</v>
       </c>
     </row>
     <row r="133">
@@ -22453,13 +22453,13 @@
         <v>0.4065040650406504</v>
       </c>
       <c r="Y133" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z133" t="b">
         <v>1</v>
       </c>
       <c r="AA133" t="n">
-        <v>0.3816155929693705</v>
+        <v>0.3821764337651064</v>
       </c>
     </row>
     <row r="134">
@@ -22540,13 +22540,13 @@
         <v>0.3731343283582089</v>
       </c>
       <c r="Y134" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z134" t="b">
         <v>1</v>
       </c>
       <c r="AA134" t="n">
-        <v>0.3462739704323217</v>
+        <v>0.3470203754218331</v>
       </c>
     </row>
     <row r="135">
@@ -22627,13 +22627,13 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="Y135" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z135" t="b">
         <v>1</v>
       </c>
       <c r="AA135" t="n">
-        <v>0.6519266379893413</v>
+        <v>0.6528847410153901</v>
       </c>
     </row>
     <row r="136">
@@ -22714,13 +22714,13 @@
         <v>0.6993006993006994</v>
       </c>
       <c r="Y136" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z136" t="b">
         <v>1</v>
       </c>
       <c r="AA136" t="n">
-        <v>0.6489610075235122</v>
+        <v>0.6503598644269322</v>
       </c>
     </row>
     <row r="137">
@@ -22801,13 +22801,13 @@
         <v>0.7874015748031495</v>
       </c>
       <c r="Y137" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z137" t="b">
         <v>1</v>
       </c>
       <c r="AA137" t="n">
-        <v>0.7391924084288594</v>
+        <v>0.740278761466269</v>
       </c>
     </row>
     <row r="138">
@@ -22888,13 +22888,13 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="Y138" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z138" t="b">
         <v>1</v>
       </c>
       <c r="AA138" t="n">
-        <v>0.7193908843090095</v>
+        <v>0.7209415551399323</v>
       </c>
     </row>
     <row r="139">
@@ -22975,13 +22975,13 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="Y139" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z139" t="b">
         <v>1</v>
       </c>
       <c r="AA139" t="n">
-        <v>0.763231185938741</v>
+        <v>0.7643528675302128</v>
       </c>
     </row>
     <row r="140">
@@ -23062,13 +23062,13 @@
         <v>0.8</v>
       </c>
       <c r="Y140" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z140" t="b">
         <v>1</v>
       </c>
       <c r="AA140" t="n">
-        <v>0.7424113926068979</v>
+        <v>0.7440116849044103</v>
       </c>
     </row>
     <row r="141">
@@ -23149,13 +23149,13 @@
         <v>0.6211180124223602</v>
       </c>
       <c r="Y141" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z141" t="b">
         <v>1</v>
       </c>
       <c r="AA141" t="n">
-        <v>0.5830896637917089</v>
+        <v>0.5839466006597277</v>
       </c>
     </row>
     <row r="142">
@@ -23236,13 +23236,13 @@
         <v>0.6134969325153374</v>
       </c>
       <c r="Y142" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z142" t="b">
         <v>1</v>
       </c>
       <c r="AA142" t="n">
-        <v>0.5693338900359647</v>
+        <v>0.5705611080555294</v>
       </c>
     </row>
     <row r="143">
@@ -23323,13 +23323,13 @@
         <v>0.8695652173913044</v>
       </c>
       <c r="Y143" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z143" t="b">
         <v>1</v>
       </c>
       <c r="AA143" t="n">
-        <v>0.8163255293083926</v>
+        <v>0.817525240923619</v>
       </c>
     </row>
     <row r="144">
@@ -23410,13 +23410,13 @@
         <v>0.8620689655172414</v>
       </c>
       <c r="Y144" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z144" t="b">
         <v>1</v>
       </c>
       <c r="AA144" t="n">
-        <v>0.8000122765160538</v>
+        <v>0.8017367294228559</v>
       </c>
     </row>
     <row r="145">
@@ -23497,13 +23497,13 @@
         <v>0.2597402597402597</v>
       </c>
       <c r="Y145" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z145" t="b">
         <v>1</v>
       </c>
       <c r="AA145" t="n">
-        <v>0.2438374957674419</v>
+        <v>0.2441958511849771</v>
       </c>
     </row>
     <row r="146">
@@ -23584,13 +23584,13 @@
         <v>0.28328611898017</v>
       </c>
       <c r="Y146" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z146" t="b">
         <v>1</v>
       </c>
       <c r="AA146" t="n">
-        <v>0.2628935526228392</v>
+        <v>0.2634602283655844</v>
       </c>
     </row>
     <row r="147">
@@ -23671,13 +23671,13 @@
         <v>0.2173913043478261</v>
       </c>
       <c r="Y147" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z147" t="b">
         <v>1</v>
       </c>
       <c r="AA147" t="n">
-        <v>0.2040813823270982</v>
+        <v>0.2043813102309048</v>
       </c>
     </row>
     <row r="148">
@@ -23750,7 +23750,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr"/>
       <c r="Y148" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z148" t="b">
         <v>1</v>
@@ -23835,13 +23835,13 @@
         <v>0.495049504950495</v>
       </c>
       <c r="Y149" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z149" t="b">
         <v>1</v>
       </c>
       <c r="AA149" t="n">
-        <v>0.4647397815369562</v>
+        <v>0.4654227856743375</v>
       </c>
     </row>
     <row r="150">
@@ -23922,13 +23922,13 @@
         <v>0.4716981132075471</v>
       </c>
       <c r="Y150" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z150" t="b">
         <v>1</v>
       </c>
       <c r="AA150" t="n">
-        <v>0.4377425663955765</v>
+        <v>0.438686134967223</v>
       </c>
     </row>
     <row r="151">
@@ -24009,13 +24009,13 @@
         <v>0.2380952380952381</v>
       </c>
       <c r="Y151" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z151" t="b">
         <v>1</v>
       </c>
       <c r="AA151" t="n">
-        <v>0.2235177044534884</v>
+        <v>0.2238461969195623</v>
       </c>
     </row>
     <row r="152">
@@ -24096,13 +24096,13 @@
         <v>0.2702702702702702</v>
       </c>
       <c r="Y152" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z152" t="b">
         <v>1</v>
       </c>
       <c r="AA152" t="n">
-        <v>0.2508146596644925</v>
+        <v>0.2513552989541926</v>
       </c>
     </row>
     <row r="153">
@@ -24183,13 +24183,13 @@
         <v>0.390625</v>
       </c>
       <c r="Y153" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z153" t="b">
         <v>1</v>
       </c>
       <c r="AA153" t="n">
-        <v>0.3667087338690045</v>
+        <v>0.3672476668211569</v>
       </c>
     </row>
     <row r="154">
@@ -24270,13 +24270,13 @@
         <v>0.4132231404958678</v>
       </c>
       <c r="Y154" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z154" t="b">
         <v>1</v>
       </c>
       <c r="AA154" t="n">
-        <v>0.3834769589911663</v>
+        <v>0.384303556252278</v>
       </c>
     </row>
     <row r="155">
@@ -24357,13 +24357,13 @@
         <v>0.4201680672268908</v>
       </c>
       <c r="Y155" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z155" t="b">
         <v>1</v>
       </c>
       <c r="AA155" t="n">
-        <v>0.3944430078590972</v>
+        <v>0.3950227004462865</v>
       </c>
     </row>
     <row r="156">
@@ -24436,7 +24436,7 @@
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr"/>
       <c r="Y156" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z156" t="b">
         <v>1</v>
@@ -24521,13 +24521,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y157" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z157" t="b">
         <v>1</v>
       </c>
       <c r="AA157" t="n">
-        <v>0.5274013251149727</v>
+        <v>0.5281764196978437</v>
       </c>
     </row>
     <row r="158">
@@ -24608,13 +24608,13 @@
         <v>0.5617977528089888</v>
       </c>
       <c r="Y158" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z158" t="b">
         <v>1</v>
       </c>
       <c r="AA158" t="n">
-        <v>0.5213563150329339</v>
+        <v>0.5224801158036589</v>
       </c>
     </row>
     <row r="159">
@@ -24695,13 +24695,13 @@
         <v>0.7751937984496123</v>
       </c>
       <c r="Y159" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z159" t="b">
         <v>1</v>
       </c>
       <c r="AA159" t="n">
-        <v>0.7277320610113577</v>
+        <v>0.7288015713660168</v>
       </c>
     </row>
     <row r="160">
@@ -24782,13 +24782,13 @@
         <v>0.3968253968253968</v>
       </c>
       <c r="Y160" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z160" t="b">
         <v>1</v>
       </c>
       <c r="AA160" t="n">
-        <v>0.3725295074224807</v>
+        <v>0.3730769948659372</v>
       </c>
     </row>
     <row r="161">
@@ -24869,13 +24869,13 @@
         <v>0.5586592178770949</v>
       </c>
       <c r="Y161" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z161" t="b">
         <v>1</v>
       </c>
       <c r="AA161" t="n">
-        <v>0.5244549489970119</v>
+        <v>0.5252257134425484</v>
       </c>
     </row>
     <row r="162">
@@ -24948,7 +24948,7 @@
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr"/>
       <c r="Y162" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z162" t="b">
         <v>1</v>
@@ -25033,13 +25033,13 @@
         <v>0.8264462809917356</v>
       </c>
       <c r="Y163" t="n">
-        <v>0.0652186978986404</v>
+        <v>0.06365549815794305</v>
       </c>
       <c r="Z163" t="b">
         <v>1</v>
       </c>
       <c r="AA163" t="n">
-        <v>0.7758465774418607</v>
+        <v>0.7769867992249271</v>
       </c>
     </row>
     <row r="164">
@@ -25120,13 +25120,13 @@
         <v>0.8130081300813008</v>
       </c>
       <c r="Y164" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z164" t="b">
         <v>1</v>
       </c>
       <c r="AA164" t="n">
-        <v>0.7544831225679857</v>
+        <v>0.7561094358784657</v>
       </c>
     </row>
     <row r="165">
@@ -25207,13 +25207,13 @@
         <v>0.2932551319648093</v>
       </c>
       <c r="Y165" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z165" t="b">
         <v>1</v>
       </c>
       <c r="AA165" t="n">
-        <v>0.2721449386388922</v>
+        <v>0.2727315560500037</v>
       </c>
     </row>
     <row r="166">
@@ -25294,13 +25294,13 @@
         <v>0.53475935828877</v>
       </c>
       <c r="Y166" t="n">
-        <v>0.07756967089484697</v>
+        <v>0.07525192981718169</v>
       </c>
       <c r="Z166" t="b">
         <v>1</v>
       </c>
       <c r="AA166" t="n">
-        <v>0.496264299870921</v>
+        <v>0.4973340139735362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>